<commit_message>
Actualizacion automatica del mapa (2026-03-10 12:20:57)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_PEBCOM.xlsx
+++ b/mapa_interactivo_PEBCOM.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,96 +413,96 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R214"/>
+  <dimension ref="A1:R222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Caso</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>F. De Reclamo</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Direccion</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Comuna</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Proveedor Asignado</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>OT</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Tipo de tarea</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Equipo</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Tipo de Elemento</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Attachments</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Coordenada_X</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Coordenada_Y</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Operacion</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Zona</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>PD</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>N2</t>
         </is>
@@ -8416,7 +8404,11 @@
           <t>ESTADOS UNIDOS 4030</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr"/>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="E94" t="inlineStr">
         <is>
           <t>Pendiente</t>
@@ -8434,8 +8426,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>base corroida
-Colocar PRFV 400</t>
+          <t>base corroida Colocar PRFV 400</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -8486,7 +8477,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve"> S01123014</t>
+          <t>S01123014</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -9174,7 +9165,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t xml:space="preserve">7981 </t>
+          <t>7981</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -9209,7 +9200,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Columna de telecom corroida en base para retira A pocos metros ya hay columna nueva de telecentro </t>
+          <t>Columna de telecom corroida en base para retira A pocos metros ya hay columna nueva de telecentro</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -9260,7 +9251,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">7874 </t>
+          <t>7874</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -9948,7 +9939,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t xml:space="preserve">7919 </t>
+          <t>7919</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -10120,7 +10111,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t xml:space="preserve">7891 </t>
+          <t>7891</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -10206,7 +10197,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 7961</t>
+          <t>7961</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -10550,7 +10541,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t xml:space="preserve">7939 </t>
+          <t>7939</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -10722,7 +10713,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t xml:space="preserve">900008939210 </t>
+          <t>900008939210</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -10894,7 +10885,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t xml:space="preserve">7929 </t>
+          <t>7929</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -10980,7 +10971,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t xml:space="preserve">7933 </t>
+          <t>7933</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -11754,7 +11745,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve"> S01199412</t>
+          <t>S01199412</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -12012,7 +12003,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">7965 </t>
+          <t>7965</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -12098,7 +12089,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">7971 </t>
+          <t>7971</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -12270,7 +12261,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">7976 </t>
+          <t>7976</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -12356,7 +12347,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">7980 </t>
+          <t>7980</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -12442,7 +12433,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">6343 </t>
+          <t>6343</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -12786,7 +12777,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">7995 </t>
+          <t>7995</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -14162,7 +14153,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t xml:space="preserve">8170 </t>
+          <t>8170</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -14248,7 +14239,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t xml:space="preserve">8123 </t>
+          <t>8123</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -14592,7 +14583,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t xml:space="preserve">8150 </t>
+          <t>8150</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -16308,7 +16299,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t xml:space="preserve">8349 </t>
+          <t>8349</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -17684,7 +17675,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>-756</t>
+          <t>8540</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -18372,7 +18363,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t xml:space="preserve">8405 </t>
+          <t>8405</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -18794,6 +18785,694 @@
         </is>
       </c>
       <c r="R214" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>S00165389</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>3/5/2026</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>HONDURAS AV. 3708</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L215" t="n">
+        <v>1</v>
+      </c>
+      <c r="M215" t="n">
+        <v>-58.414717</v>
+      </c>
+      <c r="N215" t="n">
+        <v>-34.594123</v>
+      </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P215" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q215" t="inlineStr">
+        <is>
+          <t>VCR-B</t>
+        </is>
+      </c>
+      <c r="R215" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>8509</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>3/6/2026</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>GANDHI, MAHATMA 218</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>inclinada</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>Desmonte</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>Poste</t>
+        </is>
+      </c>
+      <c r="L216" t="n">
+        <v>1</v>
+      </c>
+      <c r="M216" t="n">
+        <v>-58.440278</v>
+      </c>
+      <c r="N216" t="n">
+        <v>-34.603336</v>
+      </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P216" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q216" t="inlineStr">
+        <is>
+          <t>ALM-N</t>
+        </is>
+      </c>
+      <c r="R216" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>8514</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>3/6/2026</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAMARGO 481 </t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L217" t="n">
+        <v>1</v>
+      </c>
+      <c r="M217" t="n">
+        <v>-58.439755</v>
+      </c>
+      <c r="N217" t="n">
+        <v>-34.60075</v>
+      </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P217" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q217" t="inlineStr">
+        <is>
+          <t>VCR-J</t>
+        </is>
+      </c>
+      <c r="R217" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>900009601610</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>3/6/2026</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>THAMES 1109</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>inclinada</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L218" t="n">
+        <v>1</v>
+      </c>
+      <c r="M218" t="n">
+        <v>-58.436188</v>
+      </c>
+      <c r="N218" t="n">
+        <v>-34.59138</v>
+      </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P218" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q218" t="inlineStr">
+        <is>
+          <t>VCR-I</t>
+        </is>
+      </c>
+      <c r="R218" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>S00194756</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>3/6/2026</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>CALIFORNIA 2861</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>columna inclinada</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L219" t="n">
+        <v>1</v>
+      </c>
+      <c r="M219" t="n">
+        <v>-58.38692</v>
+      </c>
+      <c r="N219" t="n">
+        <v>-34.649509</v>
+      </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="P219" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q219" t="inlineStr">
+        <is>
+          <t>CON-I</t>
+        </is>
+      </c>
+      <c r="R219" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>8427</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>3/5/2026</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ESPINOSA 98 </t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>base quebrada</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L220" t="n">
+        <v>1</v>
+      </c>
+      <c r="M220" t="n">
+        <v>-58.446457</v>
+      </c>
+      <c r="N220" t="n">
+        <v>-34.621398</v>
+      </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P220" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q220" t="inlineStr">
+        <is>
+          <t>PCH-G</t>
+        </is>
+      </c>
+      <c r="R220" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>8483</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>3/5/2026</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>RODRIGUEZ PEÑA 1650</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L221" t="n">
+        <v>1</v>
+      </c>
+      <c r="M221" t="n">
+        <v>-58.389533</v>
+      </c>
+      <c r="N221" t="n">
+        <v>-34.591306</v>
+      </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>Recoleta</t>
+        </is>
+      </c>
+      <c r="P221" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q221" t="inlineStr">
+        <is>
+          <t>RET-L</t>
+        </is>
+      </c>
+      <c r="R221" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>8556</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>3/9/2026</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>OLAVARRIA 861</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>inclinada</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L222" t="n">
+        <v>1</v>
+      </c>
+      <c r="M222" t="n">
+        <v>-58.365014</v>
+      </c>
+      <c r="N222" t="n">
+        <v>-34.638541</v>
+      </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="P222" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q222" t="inlineStr">
+        <is>
+          <t>CON-E</t>
+        </is>
+      </c>
+      <c r="R222" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-11 15:32:33)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_PEBCOM.xlsx
+++ b/mapa_interactivo_PEBCOM.xlsx
@@ -7135,7 +7135,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Ugarteche 3075</t>
+          <t>UGARTECHE 3079</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -7995,7 +7995,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Castillo 4</t>
+          <t>CASTILLO 12</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -8042,10 +8042,10 @@
         <v>1</v>
       </c>
       <c r="M89" t="n">
-        <v>-58.430346</v>
+        <v>-58.430396</v>
       </c>
       <c r="N89" t="n">
-        <v>-34.599721</v>
+        <v>-34.599668</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
@@ -11349,7 +11349,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Catamarca 236</t>
+          <t>Catamarca 236</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-18 10:10:09)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_PEBCOM.xlsx
+++ b/mapa_interactivo_PEBCOM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R180"/>
+  <dimension ref="A1:R181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15894,6 +15894,84 @@
         </is>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" t="inlineStr"/>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>3/18/2026</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>GALLARDO, ANGEL AV. 1072</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr"/>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Reubicar columna y rienda, Angel Gallardo 1072 a 1084</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L181" t="n">
+        <v>1</v>
+      </c>
+      <c r="M181" t="n">
+        <v>-58.444908</v>
+      </c>
+      <c r="N181" t="n">
+        <v>-34.607205</v>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>ALM-O</t>
+        </is>
+      </c>
+      <c r="R181" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-04-07 12:05:53)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_PEBCOM.xlsx
+++ b/mapa_interactivo_PEBCOM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R177"/>
+  <dimension ref="A1:R178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15577,7 +15577,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G177" t="inlineStr"/>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>812879764</t>
+        </is>
+      </c>
       <c r="H177" t="inlineStr">
         <is>
           <t>Reubicar columna y rienda, Angel Gallardo 1072 a 1084</t>
@@ -15623,6 +15627,88 @@
         </is>
       </c>
       <c r="R177" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>M881</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>4/1/2026</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>AV LA PLATA 881</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr"/>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>DESMONTAR COLUMNA Y  DESPLAZAR PCALOGERO</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L178" t="n">
+        <v>1</v>
+      </c>
+      <c r="M178" t="n">
+        <v>-58.42712</v>
+      </c>
+      <c r="N178" t="n">
+        <v>-34.625871</v>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P178" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q178" t="inlineStr">
+        <is>
+          <t>ALM-A</t>
+        </is>
+      </c>
+      <c r="R178" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-04-13 10:39:19)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_PEBCOM.xlsx
+++ b/mapa_interactivo_PEBCOM.xlsx
@@ -15663,7 +15663,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G178" t="inlineStr"/>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>813046342</t>
+        </is>
+      </c>
       <c r="H178" t="inlineStr">
         <is>
           <t>DESMONTAR COLUMNA Y  DESPLAZAR PCALOGERO</t>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-04-16 09:12:44)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_PEBCOM.xlsx
+++ b/mapa_interactivo_PEBCOM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R178"/>
+  <dimension ref="A1:R177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15551,20 +15551,24 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" t="inlineStr"/>
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>M881</t>
+        </is>
+      </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>3/18/2026</t>
+          <t>4/1/2026</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>GALLARDO, ANGEL AV. 1072</t>
+          <t>AV LA PLATA 881</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
@@ -15579,12 +15583,12 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>812879764</t>
+          <t>813046342</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>Reubicar columna y rienda, Angel Gallardo 1072 a 1084</t>
+          <t>DESMONTAR COLUMNA Y  DESPLAZAR PCALOGERO</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -15606,14 +15610,14 @@
         <v>1</v>
       </c>
       <c r="M177" t="n">
-        <v>-58.444908</v>
+        <v>-58.42712</v>
       </c>
       <c r="N177" t="n">
-        <v>-34.607205</v>
+        <v>-34.625871</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P177" t="inlineStr">
@@ -15623,96 +15627,10 @@
       </c>
       <c r="Q177" t="inlineStr">
         <is>
-          <t>ALM-O</t>
+          <t>ALM-A</t>
         </is>
       </c>
       <c r="R177" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>M881</t>
-        </is>
-      </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>4/1/2026</t>
-        </is>
-      </c>
-      <c r="C178" t="inlineStr">
-        <is>
-          <t>AV LA PLATA 881</t>
-        </is>
-      </c>
-      <c r="D178" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E178" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F178" t="inlineStr">
-        <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G178" t="inlineStr">
-        <is>
-          <t>813046342</t>
-        </is>
-      </c>
-      <c r="H178" t="inlineStr">
-        <is>
-          <t>DESMONTAR COLUMNA Y  DESPLAZAR PCALOGERO</t>
-        </is>
-      </c>
-      <c r="I178" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J178" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K178" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L178" t="n">
-        <v>1</v>
-      </c>
-      <c r="M178" t="n">
-        <v>-58.42712</v>
-      </c>
-      <c r="N178" t="n">
-        <v>-34.625871</v>
-      </c>
-      <c r="O178" t="inlineStr">
-        <is>
-          <t>Boedo</t>
-        </is>
-      </c>
-      <c r="P178" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q178" t="inlineStr">
-        <is>
-          <t>ALM-A</t>
-        </is>
-      </c>
-      <c r="R178" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-05-20 09:49:42)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_PEBCOM.xlsx
+++ b/mapa_interactivo_PEBCOM.xlsx
@@ -14961,7 +14961,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>AV LA PLATA 881</t>
+          <t>AV LA PLATA 2288</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -15008,10 +15008,10 @@
         <v>1</v>
       </c>
       <c r="M170" t="n">
-        <v>-58.42712</v>
+        <v>-58.423203</v>
       </c>
       <c r="N170" t="n">
-        <v>-34.625871</v>
+        <v>-34.640909</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -15025,7 +15025,7 @@
       </c>
       <c r="Q170" t="inlineStr">
         <is>
-          <t>ALM-A</t>
+          <t>PPT-L</t>
         </is>
       </c>
       <c r="R170" t="inlineStr">

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-05-27 07:22:50)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_PEBCOM.xlsx
+++ b/mapa_interactivo_PEBCOM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R168"/>
+  <dimension ref="A1:R171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10841,22 +10841,22 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>PJ00040</t>
+          <t>LR00001</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>4/20/2026</t>
+          <t>4/27/2026</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>HONDURAS 4822</t>
+          <t>BILLINGHURST 1796</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -10871,7 +10871,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>813350536</t>
+          <t>813350523</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -10881,7 +10881,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
@@ -10898,14 +10898,14 @@
         <v>1</v>
       </c>
       <c r="M123" t="n">
-        <v>-58.428528</v>
+        <v>-58.409695</v>
       </c>
       <c r="N123" t="n">
-        <v>-34.589872</v>
+        <v>-34.589662</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P123" t="inlineStr">
@@ -10915,7 +10915,7 @@
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>VCR-F</t>
+          <t>AGU-D</t>
         </is>
       </c>
       <c r="R123" t="inlineStr">
@@ -10927,7 +10927,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>AF00001</t>
+          <t>PJ00040</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -10937,7 +10937,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>SALGUERO, JERONIMO 1995</t>
+          <t>HONDURAS 4822</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -10957,7 +10957,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>813304889</t>
+          <t>813350536</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -10967,7 +10967,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
@@ -10984,10 +10984,10 @@
         <v>1</v>
       </c>
       <c r="M124" t="n">
-        <v>-58.413378</v>
+        <v>-58.428528</v>
       </c>
       <c r="N124" t="n">
-        <v>-34.587254</v>
+        <v>-34.589872</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -11001,7 +11001,7 @@
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>VCR-G</t>
+          <t>VCR-F</t>
         </is>
       </c>
       <c r="R124" t="inlineStr">
@@ -11013,7 +11013,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>8921</t>
+          <t>AF00001</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -11023,7 +11023,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>DORREGO AV.2752</t>
+          <t>SALGUERO, JERONIMO 1995</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -11043,7 +11043,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>813305004</t>
+          <t>813304889</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -11070,10 +11070,10 @@
         <v>1</v>
       </c>
       <c r="M125" t="n">
-        <v>-58.43266</v>
+        <v>-58.413378</v>
       </c>
       <c r="N125" t="n">
-        <v>-34.574202</v>
+        <v>-34.587254</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -11087,7 +11087,7 @@
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>BLO-G</t>
+          <t>VCR-G</t>
         </is>
       </c>
       <c r="R125" t="inlineStr">
@@ -11099,22 +11099,22 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>S0000223</t>
+          <t>9006</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>4/21/2026</t>
+          <t>4/20/2026</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>ARENALES 3660</t>
+          <t>CHARCAS 3250</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -11129,7 +11129,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>813352547</t>
+          <t>813304917</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -11156,14 +11156,14 @@
         <v>1</v>
       </c>
       <c r="M126" t="n">
-        <v>-58.413732</v>
+        <v>-58.41175</v>
       </c>
       <c r="N126" t="n">
-        <v>-34.585415</v>
+        <v>-34.592173</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
@@ -11173,7 +11173,7 @@
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>AGU-L</t>
+          <t>AGU-C</t>
         </is>
       </c>
       <c r="R126" t="inlineStr">
@@ -11185,17 +11185,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>000025</t>
+          <t>8921</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>4/23/2026</t>
+          <t>4/20/2026</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>AV DORREGO 3900</t>
+          <t>DORREGO AV.2752</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -11215,12 +11215,12 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>813352568</t>
+          <t>813305004</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>POSTE CAIDO, VER POSIBILIDAD DE DESMONTE</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -11235,17 +11235,17 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L127" t="n">
         <v>1</v>
       </c>
       <c r="M127" t="n">
-        <v>-58.418801</v>
+        <v>-58.43266</v>
       </c>
       <c r="N127" t="n">
-        <v>-34.564182</v>
+        <v>-34.574202</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -11259,7 +11259,7 @@
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>BLO-?</t>
+          <t>BLO-G</t>
         </is>
       </c>
       <c r="R127" t="inlineStr">
@@ -11271,22 +11271,22 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>9025</t>
+          <t>S00419298</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>4/24/2026</t>
+          <t>4/20/2026</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>ALVAREZ, JULIAN 2552</t>
+          <t>AUSTRIA 2354</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -11301,7 +11301,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>813352603</t>
+          <t>813350615</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -11328,14 +11328,14 @@
         <v>1</v>
       </c>
       <c r="M128" t="n">
-        <v>-58.413555</v>
+        <v>-58.401523</v>
       </c>
       <c r="N128" t="n">
-        <v>-34.585955</v>
+        <v>-34.586182</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P128" t="inlineStr">
@@ -11345,7 +11345,7 @@
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>AGU-L</t>
+          <t>AGU-H</t>
         </is>
       </c>
       <c r="R128" t="inlineStr">
@@ -11357,17 +11357,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>9062</t>
+          <t>S0000223</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>4/30/2026</t>
+          <t>4/21/2026</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>BULNES 2550</t>
+          <t>ARENALES 3660</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -11387,17 +11387,17 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>813631416</t>
+          <t>813352547</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
@@ -11414,10 +11414,10 @@
         <v>1</v>
       </c>
       <c r="M129" t="n">
-        <v>-58.407013</v>
+        <v>-58.413732</v>
       </c>
       <c r="N129" t="n">
-        <v>-34.582645</v>
+        <v>-34.585415</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -11431,7 +11431,7 @@
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>AGU-N</t>
+          <t>AGU-L</t>
         </is>
       </c>
       <c r="R129" t="inlineStr">
@@ -11443,17 +11443,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>9063</t>
+          <t>000025</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>4/30/2026</t>
+          <t>4/23/2026</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>DEL LIBERTADOR AV. 2030</t>
+          <t>AV DORREGO 3900</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -11473,17 +11473,17 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>813631417</t>
+          <t>813352568</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>POSTE CAIDO, VER POSIBILIDAD DE DESMONTE</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -11493,21 +11493,21 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L130" t="n">
         <v>1</v>
       </c>
       <c r="M130" t="n">
-        <v>-58.401882</v>
+        <v>-58.418801</v>
       </c>
       <c r="N130" t="n">
-        <v>-34.582006</v>
+        <v>-34.564182</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
@@ -11517,7 +11517,7 @@
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>AGU-I</t>
+          <t>BLO-?</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
@@ -11529,17 +11529,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>9050</t>
+          <t>9025</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>4/30/2026</t>
+          <t>4/24/2026</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>CASTEX 3439</t>
+          <t>ALVAREZ, JULIAN 2552</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -11559,7 +11559,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>813631425</t>
+          <t>813352603</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -11586,10 +11586,10 @@
         <v>1</v>
       </c>
       <c r="M131" t="n">
-        <v>-58.406414</v>
+        <v>-58.413555</v>
       </c>
       <c r="N131" t="n">
-        <v>-34.577519</v>
+        <v>-34.585955</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -11603,7 +11603,7 @@
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>AGU-R</t>
+          <t>AGU-L</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
@@ -11615,7 +11615,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>9080</t>
+          <t>9062</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -11625,7 +11625,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>LACROZE, FEDERICO AV. 2338</t>
+          <t>BULNES 2550</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -11645,7 +11645,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>813631432</t>
+          <t>813631416</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -11672,24 +11672,24 @@
         <v>1</v>
       </c>
       <c r="M132" t="n">
-        <v>-58.444112</v>
+        <v>-58.407013</v>
       </c>
       <c r="N132" t="n">
-        <v>-34.569261</v>
+        <v>-34.582645</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>BLO-L</t>
+          <t>AGU-N</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
@@ -11701,7 +11701,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>9081</t>
+          <t>9063</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -11711,7 +11711,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>SOLDADO DE LA INDEPENDENCIA 1102</t>
+          <t>DEL LIBERTADOR AV. 2030</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -11731,7 +11731,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>813631446</t>
+          <t>813631417</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -11741,7 +11741,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -11758,14 +11758,14 @@
         <v>1</v>
       </c>
       <c r="M133" t="n">
-        <v>-58.438595</v>
+        <v>-58.401882</v>
       </c>
       <c r="N133" t="n">
-        <v>-34.565168</v>
+        <v>-34.582006</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
@@ -11775,7 +11775,7 @@
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>BLO-J</t>
+          <t>AGU-I</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
@@ -11787,7 +11787,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>9083</t>
+          <t>9050</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -11797,7 +11797,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ARCE 949</t>
+          <t>CASTEX 3439</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -11817,17 +11817,17 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>813631449</t>
+          <t>813631425</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -11844,10 +11844,10 @@
         <v>1</v>
       </c>
       <c r="M134" t="n">
-        <v>-58.437217</v>
+        <v>-58.406414</v>
       </c>
       <c r="N134" t="n">
-        <v>-34.567174</v>
+        <v>-34.577519</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -11861,7 +11861,7 @@
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>BLO-J</t>
+          <t>AGU-R</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
@@ -11873,7 +11873,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>9084</t>
+          <t>9080</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -11883,7 +11883,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAMPOS, LUIS M. AV. 1188 </t>
+          <t>LACROZE, FEDERICO AV. 2338</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -11903,17 +11903,17 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>813631451</t>
+          <t>813631432</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -11930,19 +11930,19 @@
         <v>1</v>
       </c>
       <c r="M135" t="n">
-        <v>-58.44018</v>
+        <v>-58.444112</v>
       </c>
       <c r="N135" t="n">
-        <v>-34.565612</v>
+        <v>-34.569261</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -11959,7 +11959,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>9085</t>
+          <t>9081</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -11969,7 +11969,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>VILLANUEVA 1212</t>
+          <t>SOLDADO DE LA INDEPENDENCIA 1102</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -11989,7 +11989,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>813631452</t>
+          <t>813631446</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -12016,24 +12016,24 @@
         <v>1</v>
       </c>
       <c r="M136" t="n">
-        <v>-58.441718</v>
+        <v>-58.438595</v>
       </c>
       <c r="N136" t="n">
-        <v>-34.566411</v>
+        <v>-34.565168</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>BLO-L</t>
+          <t>BLO-J</t>
         </is>
       </c>
       <c r="R136" t="inlineStr">
@@ -12045,7 +12045,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>9086</t>
+          <t>9083</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -12055,7 +12055,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>CAPDEVILA 3245</t>
+          <t>ARCE 949</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -12075,17 +12075,17 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>813631453</t>
+          <t>813631449</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
@@ -12102,24 +12102,24 @@
         <v>1</v>
       </c>
       <c r="M137" t="n">
-        <v>-58.492198</v>
+        <v>-58.437217</v>
       </c>
       <c r="N137" t="n">
-        <v>-34.567241</v>
+        <v>-34.567174</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>PUE-F</t>
+          <t>BLO-J</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
@@ -12131,17 +12131,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>S00432540</t>
+          <t>9084</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>4/30/2026</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>DUMONT, SANTOS 2618</t>
+          <t xml:space="preserve">CAMPOS, LUIS M. AV. 1188 </t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -12159,15 +12159,19 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G138" t="inlineStr"/>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>813631451</t>
+        </is>
+      </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
@@ -12184,10 +12188,10 @@
         <v>1</v>
       </c>
       <c r="M138" t="n">
-        <v>-58.440439</v>
+        <v>-58.44018</v>
       </c>
       <c r="N138" t="n">
-        <v>-34.575416</v>
+        <v>-34.565612</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -12201,7 +12205,7 @@
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>COG-B</t>
+          <t>BLO-L</t>
         </is>
       </c>
       <c r="R138" t="inlineStr">
@@ -12213,17 +12217,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">9180 </t>
+          <t>9085</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>4/30/2026</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>MIGUELETES 1156</t>
+          <t>VILLANUEVA 1212</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -12241,15 +12245,19 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G139" t="inlineStr"/>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>813631452</t>
+        </is>
+      </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -12266,24 +12274,24 @@
         <v>1</v>
       </c>
       <c r="M139" t="n">
-        <v>-58.438274</v>
+        <v>-58.441718</v>
       </c>
       <c r="N139" t="n">
-        <v>-34.564049</v>
+        <v>-34.566411</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>BLO-J</t>
+          <t>BLO-L</t>
         </is>
       </c>
       <c r="R139" t="inlineStr">
@@ -12295,22 +12303,22 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">9115 </t>
+          <t>9086</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>4/30/2026</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>NEWBERY, JORGE 1694</t>
+          <t>CAPDEVILA 3245</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
@@ -12323,7 +12331,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G140" t="inlineStr"/>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>813631453</t>
+        </is>
+      </c>
       <c r="H140" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -12348,24 +12360,24 @@
         <v>1</v>
       </c>
       <c r="M140" t="n">
-        <v>-58.434721</v>
+        <v>-58.492198</v>
       </c>
       <c r="N140" t="n">
         <v>-34.567241</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>BLO-H</t>
+          <t>PUE-F</t>
         </is>
       </c>
       <c r="R140" t="inlineStr">
@@ -12377,22 +12389,22 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">9116 </t>
+          <t>S00477293</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/10/2026</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>GOROSTIAGA 1514</t>
+          <t xml:space="preserve"> ARENALES 2552</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -12405,7 +12417,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G141" t="inlineStr"/>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>813631921</t>
+        </is>
+      </c>
       <c r="H141" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -12430,14 +12446,14 @@
         <v>1</v>
       </c>
       <c r="M141" t="n">
-        <v>-58.435738</v>
+        <v>-58.402534</v>
       </c>
       <c r="N141" t="n">
-        <v>-34.564606</v>
+        <v>-34.593133</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P141" t="inlineStr">
@@ -12447,7 +12463,7 @@
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>BLO-J</t>
+          <t>AGU-F</t>
         </is>
       </c>
       <c r="R141" t="inlineStr">
@@ -12459,7 +12475,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">9117 </t>
+          <t>S01385955</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -12469,12 +12485,12 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>MAURE 1590</t>
+          <t>POSADAS 1391</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -12490,7 +12506,7 @@
       <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA, POSIBLE NUEVA ALEDAÑA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -12512,14 +12528,14 @@
         <v>1</v>
       </c>
       <c r="M142" t="n">
-        <v>-58.435011</v>
+        <v>-58.385947</v>
       </c>
       <c r="N142" t="n">
-        <v>-34.56566</v>
+        <v>-34.588156</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P142" t="inlineStr">
@@ -12529,7 +12545,7 @@
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>BLO-J</t>
+          <t>RET-L</t>
         </is>
       </c>
       <c r="R142" t="inlineStr">
@@ -12541,7 +12557,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">9118 </t>
+          <t>S00432540</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -12551,7 +12567,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>ORTEGA Y GASSET 1590</t>
+          <t>DUMONT, SANTOS 2618</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -12572,17 +12588,17 @@
       <c r="G143" t="inlineStr"/>
       <c r="H143" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -12594,10 +12610,10 @@
         <v>1</v>
       </c>
       <c r="M143" t="n">
-        <v>-58.430774</v>
+        <v>-58.440439</v>
       </c>
       <c r="N143" t="n">
-        <v>-34.568179</v>
+        <v>-34.575416</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -12611,7 +12627,7 @@
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>BLO-I</t>
+          <t>COG-B</t>
         </is>
       </c>
       <c r="R143" t="inlineStr">
@@ -12623,7 +12639,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>9120</t>
+          <t xml:space="preserve">9180 </t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -12633,7 +12649,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>ARCE 867</t>
+          <t>MIGUELETES 1156</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -12676,10 +12692,10 @@
         <v>1</v>
       </c>
       <c r="M144" t="n">
-        <v>-58.436255</v>
+        <v>-58.438274</v>
       </c>
       <c r="N144" t="n">
-        <v>-34.567733</v>
+        <v>-34.564049</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -12705,7 +12721,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">9193 </t>
+          <t xml:space="preserve">9115 </t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -12715,7 +12731,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>CRAMER 315</t>
+          <t>NEWBERY, JORGE 1694</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -12758,10 +12774,10 @@
         <v>1</v>
       </c>
       <c r="M145" t="n">
-        <v>-58.443403</v>
+        <v>-58.434721</v>
       </c>
       <c r="N145" t="n">
-        <v>-34.575666</v>
+        <v>-34.567241</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -12775,7 +12791,7 @@
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>ATH-B</t>
+          <t>BLO-H</t>
         </is>
       </c>
       <c r="R145" t="inlineStr">
@@ -12787,7 +12803,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">9199 </t>
+          <t xml:space="preserve">9116 </t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -12797,7 +12813,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>ARMENIA 1553</t>
+          <t>GOROSTIAGA 1514</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -12840,10 +12856,10 @@
         <v>1</v>
       </c>
       <c r="M146" t="n">
-        <v>-58.428639</v>
+        <v>-58.435738</v>
       </c>
       <c r="N146" t="n">
-        <v>-34.59039</v>
+        <v>-34.564606</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -12857,7 +12873,7 @@
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>VCR-F</t>
+          <t>BLO-J</t>
         </is>
       </c>
       <c r="R146" t="inlineStr">
@@ -12869,7 +12885,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>S00522384</t>
+          <t xml:space="preserve">9117 </t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -12879,7 +12895,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>FRAY JUSTO SANTAMARIA DE ORO 2734</t>
+          <t>MAURE 1590</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -12900,7 +12916,7 @@
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA, POSIBLE NUEVA ALEDAÑA</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -12910,7 +12926,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -12922,10 +12938,10 @@
         <v>1</v>
       </c>
       <c r="M147" t="n">
-        <v>-58.422183</v>
+        <v>-58.435011</v>
       </c>
       <c r="N147" t="n">
-        <v>-34.576849</v>
+        <v>-34.56566</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -12939,7 +12955,7 @@
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>VCR-M</t>
+          <t>BLO-J</t>
         </is>
       </c>
       <c r="R147" t="inlineStr">
@@ -12951,7 +12967,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t xml:space="preserve">9220 </t>
+          <t xml:space="preserve">9118 </t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -12961,7 +12977,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>ARMENIA 1829</t>
+          <t>ORTEGA Y GASSET 1590</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -12992,7 +13008,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -13004,10 +13020,10 @@
         <v>1</v>
       </c>
       <c r="M148" t="n">
-        <v>-58.425803</v>
+        <v>-58.430774</v>
       </c>
       <c r="N148" t="n">
-        <v>-34.588513</v>
+        <v>-34.568179</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -13021,7 +13037,7 @@
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>VCR-K</t>
+          <t>BLO-I</t>
         </is>
       </c>
       <c r="R148" t="inlineStr">
@@ -13033,17 +13049,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t xml:space="preserve">10033 </t>
+          <t>9120</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>ESTADO DE PALESTINA 1192</t>
+          <t>ARCE 867</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -13064,17 +13080,17 @@
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -13086,10 +13102,10 @@
         <v>1</v>
       </c>
       <c r="M149" t="n">
-        <v>-58.424388</v>
+        <v>-58.436255</v>
       </c>
       <c r="N149" t="n">
-        <v>-34.59632</v>
+        <v>-34.567733</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -13103,7 +13119,7 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>VCR-D</t>
+          <t>BLO-J</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">
@@ -13115,17 +13131,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t xml:space="preserve">9157 </t>
+          <t xml:space="preserve">9193 </t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>GUATEMALA 5078</t>
+          <t>CRAMER 315</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -13168,10 +13184,10 @@
         <v>1</v>
       </c>
       <c r="M150" t="n">
-        <v>-58.427895</v>
+        <v>-58.443403</v>
       </c>
       <c r="N150" t="n">
-        <v>-34.583677</v>
+        <v>-34.575666</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -13185,7 +13201,7 @@
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>VCR-P</t>
+          <t>ATH-B</t>
         </is>
       </c>
       <c r="R150" t="inlineStr">
@@ -13197,17 +13213,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t xml:space="preserve">9924 </t>
+          <t xml:space="preserve">9199 </t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>CORDOBA AV. 4089</t>
+          <t>ARMENIA 1553</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -13250,10 +13266,10 @@
         <v>1</v>
       </c>
       <c r="M151" t="n">
-        <v>-58.424553</v>
+        <v>-58.428639</v>
       </c>
       <c r="N151" t="n">
-        <v>-34.59709</v>
+        <v>-34.59039</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -13267,7 +13283,7 @@
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>VCR-D</t>
+          <t>VCR-F</t>
         </is>
       </c>
       <c r="R151" t="inlineStr">
@@ -13279,22 +13295,22 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t xml:space="preserve">10047 </t>
+          <t>S00497843</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>NEWBERY, JORGE 2410</t>
+          <t>MANSILLA, LUCIO NORBERTO, GENERAL 2610</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -13310,12 +13326,12 @@
       <c r="G152" t="inlineStr"/>
       <c r="H152" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
@@ -13332,14 +13348,14 @@
         <v>1</v>
       </c>
       <c r="M152" t="n">
-        <v>-58.440973</v>
+        <v>-58.404726</v>
       </c>
       <c r="N152" t="n">
-        <v>-34.572415</v>
+        <v>-34.596069</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P152" t="inlineStr">
@@ -13349,7 +13365,7 @@
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>COG-B</t>
+          <t>AGU-A</t>
         </is>
       </c>
       <c r="R152" t="inlineStr">
@@ -13361,17 +13377,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t xml:space="preserve">10042 </t>
+          <t>S00522384</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>PARAGUAY 5310</t>
+          <t>FRAY JUSTO SANTAMARIA DE ORO 2734</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -13402,7 +13418,7 @@
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -13414,10 +13430,10 @@
         <v>1</v>
       </c>
       <c r="M153" t="n">
-        <v>-58.43218</v>
+        <v>-58.422183</v>
       </c>
       <c r="N153" t="n">
-        <v>-34.578546</v>
+        <v>-34.576849</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -13431,7 +13447,7 @@
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>ATH-B</t>
+          <t>VCR-M</t>
         </is>
       </c>
       <c r="R153" t="inlineStr">
@@ -13443,17 +13459,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t xml:space="preserve">10062 </t>
+          <t xml:space="preserve">9220 </t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>HUMBOLDT 1556</t>
+          <t>ARMENIA 1829</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -13496,10 +13512,10 @@
         <v>1</v>
       </c>
       <c r="M154" t="n">
-        <v>-58.436737</v>
+        <v>-58.425803</v>
       </c>
       <c r="N154" t="n">
-        <v>-34.58597</v>
+        <v>-34.588513</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -13513,7 +13529,7 @@
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>ATH-M</t>
+          <t>VCR-K</t>
         </is>
       </c>
       <c r="R154" t="inlineStr">
@@ -13525,7 +13541,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t xml:space="preserve">10066 </t>
+          <t xml:space="preserve">10033 </t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -13535,7 +13551,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARENALES 3640 </t>
+          <t>ESTADO DE PALESTINA 1192</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -13556,17 +13572,17 @@
       <c r="G155" t="inlineStr"/>
       <c r="H155" t="inlineStr">
         <is>
-          <t>DESMONTAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -13578,10 +13594,10 @@
         <v>1</v>
       </c>
       <c r="M155" t="n">
-        <v>-58.413584</v>
+        <v>-58.424388</v>
       </c>
       <c r="N155" t="n">
-        <v>-34.58551</v>
+        <v>-34.59632</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -13595,7 +13611,7 @@
       </c>
       <c r="Q155" t="inlineStr">
         <is>
-          <t>AGU-L</t>
+          <t>VCR-D</t>
         </is>
       </c>
       <c r="R155" t="inlineStr">
@@ -13607,7 +13623,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t xml:space="preserve">10067 </t>
+          <t xml:space="preserve">9157 </t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -13617,7 +13633,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>CHARCAS 3601</t>
+          <t>GUATEMALA 5078</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -13638,17 +13654,17 @@
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -13660,10 +13676,10 @@
         <v>1</v>
       </c>
       <c r="M156" t="n">
-        <v>-58.415912</v>
+        <v>-58.427895</v>
       </c>
       <c r="N156" t="n">
-        <v>-34.588977</v>
+        <v>-34.583677</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -13677,7 +13693,7 @@
       </c>
       <c r="Q156" t="inlineStr">
         <is>
-          <t>VCR-E</t>
+          <t>VCR-P</t>
         </is>
       </c>
       <c r="R156" t="inlineStr">
@@ -13689,7 +13705,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t xml:space="preserve">10072 </t>
+          <t xml:space="preserve">9924 </t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -13699,7 +13715,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>SANTA FE AV. 3470</t>
+          <t>CORDOBA AV. 4089</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -13720,12 +13736,12 @@
       <c r="G157" t="inlineStr"/>
       <c r="H157" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
@@ -13742,10 +13758,10 @@
         <v>1</v>
       </c>
       <c r="M157" t="n">
-        <v>-58.413885</v>
+        <v>-58.424553</v>
       </c>
       <c r="N157" t="n">
-        <v>-34.586628</v>
+        <v>-34.59709</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -13759,7 +13775,7 @@
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t>VCR-G</t>
+          <t>VCR-D</t>
         </is>
       </c>
       <c r="R157" t="inlineStr">
@@ -13771,7 +13787,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t xml:space="preserve">10080 </t>
+          <t xml:space="preserve">10047 </t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -13781,7 +13797,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>THAMES 549</t>
+          <t>NEWBERY, JORGE 2410</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -13824,10 +13840,10 @@
         <v>1</v>
       </c>
       <c r="M158" t="n">
-        <v>-58.442534</v>
+        <v>-58.440973</v>
       </c>
       <c r="N158" t="n">
-        <v>-34.59499</v>
+        <v>-34.572415</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -13841,7 +13857,7 @@
       </c>
       <c r="Q158" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>COG-B</t>
         </is>
       </c>
       <c r="R158" t="inlineStr">
@@ -13853,7 +13869,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t xml:space="preserve">10083 </t>
+          <t>S01035299</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -13863,12 +13879,12 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>ORTIZ DE OCAMPO 2639</t>
+          <t>ECUADOR 1390</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
@@ -13894,7 +13910,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -13906,10 +13922,10 @@
         <v>1</v>
       </c>
       <c r="M159" t="n">
-        <v>-58.404652</v>
+        <v>-58.40382</v>
       </c>
       <c r="N159" t="n">
-        <v>-34.58263</v>
+        <v>-34.594385</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -13923,7 +13939,7 @@
       </c>
       <c r="Q159" t="inlineStr">
         <is>
-          <t>AGU-N</t>
+          <t>AGU-A</t>
         </is>
       </c>
       <c r="R159" t="inlineStr">
@@ -13935,7 +13951,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t xml:space="preserve">10098 </t>
+          <t xml:space="preserve">10042 </t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -13945,7 +13961,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>DORREGO AV. 2635</t>
+          <t>PARAGUAY 5310</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -13988,10 +14004,10 @@
         <v>1</v>
       </c>
       <c r="M160" t="n">
-        <v>-58.433857</v>
+        <v>-58.43218</v>
       </c>
       <c r="N160" t="n">
-        <v>-34.57424</v>
+        <v>-34.578546</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -14005,7 +14021,7 @@
       </c>
       <c r="Q160" t="inlineStr">
         <is>
-          <t>BLO-G</t>
+          <t>ATH-B</t>
         </is>
       </c>
       <c r="R160" t="inlineStr">
@@ -14017,7 +14033,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t xml:space="preserve">10102 </t>
+          <t xml:space="preserve">10062 </t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -14027,7 +14043,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>ELCANO AV. 3950</t>
+          <t>HUMBOLDT 1556</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -14048,7 +14064,7 @@
       <c r="G161" t="inlineStr"/>
       <c r="H161" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -14070,24 +14086,24 @@
         <v>1</v>
       </c>
       <c r="M161" t="n">
-        <v>-58.460457</v>
+        <v>-58.436737</v>
       </c>
       <c r="N161" t="n">
-        <v>-34.582381</v>
+        <v>-34.58597</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P161" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q161" t="inlineStr">
         <is>
-          <t>ATH-H</t>
+          <t>ATH-M</t>
         </is>
       </c>
       <c r="R161" t="inlineStr">
@@ -14099,7 +14115,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t xml:space="preserve">10103 </t>
+          <t xml:space="preserve">10066 </t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -14109,7 +14125,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>DORREGO AV. 2765</t>
+          <t xml:space="preserve">ARENALES 3640 </t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -14130,12 +14146,12 @@
       <c r="G162" t="inlineStr"/>
       <c r="H162" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>DESMONTAR COLUMNA</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
@@ -14152,10 +14168,10 @@
         <v>1</v>
       </c>
       <c r="M162" t="n">
-        <v>-58.432319</v>
+        <v>-58.413584</v>
       </c>
       <c r="N162" t="n">
-        <v>-34.574385</v>
+        <v>-34.58551</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -14169,7 +14185,7 @@
       </c>
       <c r="Q162" t="inlineStr">
         <is>
-          <t>BLO-G</t>
+          <t>AGU-L</t>
         </is>
       </c>
       <c r="R162" t="inlineStr">
@@ -14181,7 +14197,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t xml:space="preserve">10104 </t>
+          <t xml:space="preserve">10067 </t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -14191,7 +14207,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t xml:space="preserve">DORREGO AV. 4050 </t>
+          <t>CHARCAS 3601</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -14212,17 +14228,17 @@
       <c r="G163" t="inlineStr"/>
       <c r="H163" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAMBIAR COLUMNA </t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -14234,10 +14250,10 @@
         <v>1</v>
       </c>
       <c r="M163" t="n">
-        <v>-58.416882</v>
+        <v>-58.415912</v>
       </c>
       <c r="N163" t="n">
-        <v>-34.562655</v>
+        <v>-34.588977</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -14251,7 +14267,7 @@
       </c>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>BLO-?</t>
+          <t>VCR-E</t>
         </is>
       </c>
       <c r="R163" t="inlineStr">
@@ -14263,7 +14279,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t xml:space="preserve">10131 </t>
+          <t xml:space="preserve">10072 </t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -14273,7 +14289,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t xml:space="preserve">PARAGUAY 4022 </t>
+          <t>SANTA FE AV. 3470</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -14294,17 +14310,17 @@
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -14316,10 +14332,10 @@
         <v>1</v>
       </c>
       <c r="M164" t="n">
-        <v>-58.419652</v>
+        <v>-58.413885</v>
       </c>
       <c r="N164" t="n">
-        <v>-34.588271</v>
+        <v>-34.586628</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -14333,7 +14349,7 @@
       </c>
       <c r="Q164" t="inlineStr">
         <is>
-          <t>VCR-K</t>
+          <t>VCR-G</t>
         </is>
       </c>
       <c r="R164" t="inlineStr">
@@ -14345,22 +14361,22 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>4512</t>
+          <t xml:space="preserve">10080 </t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>5/26/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>RIVADAVIA AV. 4512</t>
+          <t>THAMES 549</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
@@ -14373,19 +14389,15 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G165" t="inlineStr">
-        <is>
-          <t>813649670</t>
-        </is>
-      </c>
+      <c r="G165" t="inlineStr"/>
       <c r="H165" t="inlineStr">
         <is>
-          <t>REALIZAR DESPLAZAMIENTO TRAMBUS</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
@@ -14402,14 +14414,14 @@
         <v>1</v>
       </c>
       <c r="M165" t="n">
-        <v>-58.429509</v>
+        <v>-58.442534</v>
       </c>
       <c r="N165" t="n">
-        <v>-34.615307</v>
+        <v>-34.59499</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P165" t="inlineStr">
@@ -14419,7 +14431,7 @@
       </c>
       <c r="Q165" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R165" t="inlineStr">
@@ -14431,22 +14443,22 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>5027</t>
+          <t xml:space="preserve">10083 </t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>5/26/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>RIVADAVIA AV. 5012</t>
+          <t>ORTIZ DE OCAMPO 2639</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
@@ -14462,12 +14474,12 @@
       <c r="G166" t="inlineStr"/>
       <c r="H166" t="inlineStr">
         <is>
-          <t>DESPLAZAR COLUMNA TRAMBUS</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
@@ -14484,14 +14496,14 @@
         <v>1</v>
       </c>
       <c r="M166" t="n">
-        <v>-58.436804</v>
+        <v>-58.404652</v>
       </c>
       <c r="N166" t="n">
-        <v>-34.618542</v>
+        <v>-34.58263</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P166" t="inlineStr">
@@ -14501,7 +14513,7 @@
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>ALM-F</t>
+          <t>AGU-N</t>
         </is>
       </c>
       <c r="R166" t="inlineStr">
@@ -14513,22 +14525,22 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>-4992</t>
+          <t xml:space="preserve">10098 </t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>5/26/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>BEYROUTH 4992</t>
+          <t>DORREGO AV. 2635</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
@@ -14544,7 +14556,7 @@
       <c r="G167" t="inlineStr"/>
       <c r="H167" t="inlineStr">
         <is>
-          <t>REALIZAR CAMBIO DE POSTE POR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -14563,27 +14575,27 @@
         </is>
       </c>
       <c r="L167" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M167" t="n">
-        <v>-58.502223</v>
+        <v>-58.433857</v>
       </c>
       <c r="N167" t="n">
-        <v>-34.626887</v>
+        <v>-34.57424</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P167" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q167" t="inlineStr">
         <is>
-          <t>DEV-H</t>
+          <t>BLO-G</t>
         </is>
       </c>
       <c r="R167" t="inlineStr">
@@ -14595,22 +14607,22 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>-4926</t>
+          <t xml:space="preserve">10102 </t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>5/26/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>BEYROUTH 4926</t>
+          <t>ELCANO AV. 3950</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
@@ -14626,7 +14638,7 @@
       <c r="G168" t="inlineStr"/>
       <c r="H168" t="inlineStr">
         <is>
-          <t>CAMBIAR POSTE POR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -14648,14 +14660,14 @@
         <v>1</v>
       </c>
       <c r="M168" t="n">
-        <v>-58.501459</v>
+        <v>-58.460457</v>
       </c>
       <c r="N168" t="n">
-        <v>-34.626196</v>
+        <v>-34.582381</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P168" t="inlineStr">
@@ -14665,10 +14677,256 @@
       </c>
       <c r="Q168" t="inlineStr">
         <is>
-          <t>DEV-H</t>
+          <t>ATH-H</t>
         </is>
       </c>
       <c r="R168" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10103 </t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>5/14/2026</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>DORREGO AV. 2765</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr"/>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>COLUMNA INCLINADA</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L169" t="n">
+        <v>1</v>
+      </c>
+      <c r="M169" t="n">
+        <v>-58.432319</v>
+      </c>
+      <c r="N169" t="n">
+        <v>-34.574385</v>
+      </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P169" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q169" t="inlineStr">
+        <is>
+          <t>BLO-G</t>
+        </is>
+      </c>
+      <c r="R169" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10104 </t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>5/14/2026</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DORREGO AV. 4050 </t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr"/>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAMBIAR COLUMNA </t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L170" t="n">
+        <v>1</v>
+      </c>
+      <c r="M170" t="n">
+        <v>-58.416882</v>
+      </c>
+      <c r="N170" t="n">
+        <v>-34.562655</v>
+      </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P170" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q170" t="inlineStr">
+        <is>
+          <t>BLO-?</t>
+        </is>
+      </c>
+      <c r="R170" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10131 </t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>5/14/2026</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PARAGUAY 4022 </t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr"/>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>Nodo/Fuente Teco</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L171" t="n">
+        <v>1</v>
+      </c>
+      <c r="M171" t="n">
+        <v>-58.419652</v>
+      </c>
+      <c r="N171" t="n">
+        <v>-34.588271</v>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P171" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q171" t="inlineStr">
+        <is>
+          <t>VCR-K</t>
+        </is>
+      </c>
+      <c r="R171" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-05-28 07:54:41)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_PEBCOM.xlsx
+++ b/mapa_interactivo_PEBCOM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R157"/>
+  <dimension ref="A1:R159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11483,7 +11483,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t xml:space="preserve">9180 </t>
+          <t xml:space="preserve">9179 </t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -11493,7 +11493,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>MIGUELETES 1156</t>
+          <t>ARAOZ 2289</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -11536,10 +11536,10 @@
         <v>1</v>
       </c>
       <c r="M130" t="n">
-        <v>-58.438274</v>
+        <v>-58.418131</v>
       </c>
       <c r="N130" t="n">
-        <v>-34.564049</v>
+        <v>-34.58774</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -11553,7 +11553,7 @@
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>BLO-J</t>
+          <t>VCR-G</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
@@ -11565,7 +11565,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t xml:space="preserve">9115 </t>
+          <t xml:space="preserve">9180 </t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -11575,7 +11575,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>NEWBERY, JORGE 1694</t>
+          <t>MIGUELETES 1156</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -11618,10 +11618,10 @@
         <v>1</v>
       </c>
       <c r="M131" t="n">
-        <v>-58.434721</v>
+        <v>-58.438274</v>
       </c>
       <c r="N131" t="n">
-        <v>-34.567241</v>
+        <v>-34.564049</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -11635,7 +11635,7 @@
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>BLO-H</t>
+          <t>BLO-J</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
@@ -11647,7 +11647,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t xml:space="preserve">9116 </t>
+          <t xml:space="preserve">9115 </t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -11657,7 +11657,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>GOROSTIAGA 1514</t>
+          <t>NEWBERY, JORGE 1694</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -11700,10 +11700,10 @@
         <v>1</v>
       </c>
       <c r="M132" t="n">
-        <v>-58.435738</v>
+        <v>-58.434721</v>
       </c>
       <c r="N132" t="n">
-        <v>-34.564606</v>
+        <v>-34.567241</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -11717,7 +11717,7 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>BLO-J</t>
+          <t>BLO-H</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
@@ -11729,7 +11729,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">9117 </t>
+          <t xml:space="preserve">9116 </t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -11739,7 +11739,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>MAURE 1590</t>
+          <t>GOROSTIAGA 1514</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -11760,7 +11760,7 @@
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA, POSIBLE NUEVA ALEDAÑA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -11782,10 +11782,10 @@
         <v>1</v>
       </c>
       <c r="M133" t="n">
-        <v>-58.435011</v>
+        <v>-58.435738</v>
       </c>
       <c r="N133" t="n">
-        <v>-34.56566</v>
+        <v>-34.564606</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -11811,7 +11811,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">9118 </t>
+          <t xml:space="preserve">9117 </t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -11821,7 +11821,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ORTEGA Y GASSET 1590</t>
+          <t>MAURE 1590</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -11842,7 +11842,7 @@
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA, POSIBLE NUEVA ALEDAÑA</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -11852,7 +11852,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -11864,10 +11864,10 @@
         <v>1</v>
       </c>
       <c r="M134" t="n">
-        <v>-58.430774</v>
+        <v>-58.435011</v>
       </c>
       <c r="N134" t="n">
-        <v>-34.568179</v>
+        <v>-34.56566</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -11881,7 +11881,7 @@
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>BLO-I</t>
+          <t>BLO-J</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
@@ -11893,7 +11893,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>9120</t>
+          <t xml:space="preserve">9118 </t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -11903,7 +11903,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ARCE 867</t>
+          <t>ORTEGA Y GASSET 1590</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -11934,7 +11934,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -11946,10 +11946,10 @@
         <v>1</v>
       </c>
       <c r="M135" t="n">
-        <v>-58.436255</v>
+        <v>-58.430774</v>
       </c>
       <c r="N135" t="n">
-        <v>-34.567733</v>
+        <v>-34.568179</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -11963,7 +11963,7 @@
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>BLO-J</t>
+          <t>BLO-I</t>
         </is>
       </c>
       <c r="R135" t="inlineStr">
@@ -11975,7 +11975,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">9193 </t>
+          <t>9120</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -11985,7 +11985,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>CRAMER 315</t>
+          <t>ARCE 867</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -12028,10 +12028,10 @@
         <v>1</v>
       </c>
       <c r="M136" t="n">
-        <v>-58.443403</v>
+        <v>-58.436255</v>
       </c>
       <c r="N136" t="n">
-        <v>-34.575666</v>
+        <v>-34.567733</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -12045,7 +12045,7 @@
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>ATH-B</t>
+          <t>BLO-J</t>
         </is>
       </c>
       <c r="R136" t="inlineStr">
@@ -12057,7 +12057,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">9199 </t>
+          <t xml:space="preserve">9193 </t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -12067,7 +12067,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>ARMENIA 1553</t>
+          <t>CRAMER 315</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -12110,10 +12110,10 @@
         <v>1</v>
       </c>
       <c r="M137" t="n">
-        <v>-58.428639</v>
+        <v>-58.443403</v>
       </c>
       <c r="N137" t="n">
-        <v>-34.59039</v>
+        <v>-34.575666</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -12127,7 +12127,7 @@
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>VCR-F</t>
+          <t>ATH-B</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
@@ -12139,7 +12139,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>S00497843</t>
+          <t xml:space="preserve">9199 </t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -12149,12 +12149,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>MANSILLA, LUCIO NORBERTO, GENERAL 2610</t>
+          <t>ARMENIA 1553</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -12192,14 +12192,14 @@
         <v>1</v>
       </c>
       <c r="M138" t="n">
-        <v>-58.404726</v>
+        <v>-58.428639</v>
       </c>
       <c r="N138" t="n">
-        <v>-34.596069</v>
+        <v>-34.59039</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P138" t="inlineStr">
@@ -12209,7 +12209,7 @@
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>AGU-A</t>
+          <t>VCR-F</t>
         </is>
       </c>
       <c r="R138" t="inlineStr">
@@ -12221,7 +12221,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>S00522384</t>
+          <t>S00497843</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -12231,12 +12231,12 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>FRAY JUSTO SANTAMARIA DE ORO 2734</t>
+          <t>MANSILLA, LUCIO NORBERTO, GENERAL 2610</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -12262,7 +12262,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -12274,14 +12274,14 @@
         <v>1</v>
       </c>
       <c r="M139" t="n">
-        <v>-58.422183</v>
+        <v>-58.404726</v>
       </c>
       <c r="N139" t="n">
-        <v>-34.576849</v>
+        <v>-34.596069</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
@@ -12291,7 +12291,7 @@
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>VCR-M</t>
+          <t>AGU-A</t>
         </is>
       </c>
       <c r="R139" t="inlineStr">
@@ -12303,7 +12303,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">9220 </t>
+          <t>S00522384</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -12313,7 +12313,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>ARMENIA 1829</t>
+          <t>FRAY JUSTO SANTAMARIA DE ORO 2734</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -12344,7 +12344,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -12356,10 +12356,10 @@
         <v>1</v>
       </c>
       <c r="M140" t="n">
-        <v>-58.425803</v>
+        <v>-58.422183</v>
       </c>
       <c r="N140" t="n">
-        <v>-34.588513</v>
+        <v>-34.576849</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -12373,7 +12373,7 @@
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>VCR-K</t>
+          <t>VCR-M</t>
         </is>
       </c>
       <c r="R140" t="inlineStr">
@@ -12385,17 +12385,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">10033 </t>
+          <t xml:space="preserve">9220 </t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>ESTADO DE PALESTINA 1192</t>
+          <t>ARMENIA 1829</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -12416,17 +12416,17 @@
       <c r="G141" t="inlineStr"/>
       <c r="H141" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -12438,10 +12438,10 @@
         <v>1</v>
       </c>
       <c r="M141" t="n">
-        <v>-58.424388</v>
+        <v>-58.425803</v>
       </c>
       <c r="N141" t="n">
-        <v>-34.59632</v>
+        <v>-34.588513</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -12455,7 +12455,7 @@
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>VCR-D</t>
+          <t>VCR-K</t>
         </is>
       </c>
       <c r="R141" t="inlineStr">
@@ -12467,7 +12467,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">9157 </t>
+          <t xml:space="preserve">10033 </t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -12477,7 +12477,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>GUATEMALA 5078</t>
+          <t>ESTADO DE PALESTINA 1192</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -12498,17 +12498,17 @@
       <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -12520,10 +12520,10 @@
         <v>1</v>
       </c>
       <c r="M142" t="n">
-        <v>-58.427895</v>
+        <v>-58.424388</v>
       </c>
       <c r="N142" t="n">
-        <v>-34.583677</v>
+        <v>-34.59632</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -12537,7 +12537,7 @@
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>VCR-P</t>
+          <t>VCR-D</t>
         </is>
       </c>
       <c r="R142" t="inlineStr">
@@ -12549,7 +12549,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">9924 </t>
+          <t xml:space="preserve">9157 </t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -12559,7 +12559,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>CORDOBA AV. 4089</t>
+          <t>GUATEMALA 5078</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -12602,10 +12602,10 @@
         <v>1</v>
       </c>
       <c r="M143" t="n">
-        <v>-58.424553</v>
+        <v>-58.427895</v>
       </c>
       <c r="N143" t="n">
-        <v>-34.59709</v>
+        <v>-34.583677</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -12619,7 +12619,7 @@
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>VCR-D</t>
+          <t>VCR-P</t>
         </is>
       </c>
       <c r="R143" t="inlineStr">
@@ -12631,7 +12631,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">10047 </t>
+          <t xml:space="preserve">9924 </t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -12641,7 +12641,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>NEWBERY, JORGE 2410</t>
+          <t>CORDOBA AV. 4089</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -12662,12 +12662,12 @@
       <c r="G144" t="inlineStr"/>
       <c r="H144" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
@@ -12684,10 +12684,10 @@
         <v>1</v>
       </c>
       <c r="M144" t="n">
-        <v>-58.440973</v>
+        <v>-58.424553</v>
       </c>
       <c r="N144" t="n">
-        <v>-34.572415</v>
+        <v>-34.59709</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -12701,7 +12701,7 @@
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>COG-B</t>
+          <t>VCR-D</t>
         </is>
       </c>
       <c r="R144" t="inlineStr">
@@ -12713,7 +12713,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>S01035299</t>
+          <t xml:space="preserve">10047 </t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -12723,12 +12723,12 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>ECUADOR 1390</t>
+          <t>NEWBERY, JORGE 2410</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -12754,7 +12754,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -12766,14 +12766,14 @@
         <v>1</v>
       </c>
       <c r="M145" t="n">
-        <v>-58.40382</v>
+        <v>-58.440973</v>
       </c>
       <c r="N145" t="n">
-        <v>-34.594385</v>
+        <v>-34.572415</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P145" t="inlineStr">
@@ -12783,7 +12783,7 @@
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>AGU-A</t>
+          <t>COG-B</t>
         </is>
       </c>
       <c r="R145" t="inlineStr">
@@ -12795,7 +12795,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">10042 </t>
+          <t>S01035299</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -12805,12 +12805,12 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>PARAGUAY 5310</t>
+          <t>ECUADOR 1390</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -12826,17 +12826,17 @@
       <c r="G146" t="inlineStr"/>
       <c r="H146" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -12848,14 +12848,14 @@
         <v>1</v>
       </c>
       <c r="M146" t="n">
-        <v>-58.43218</v>
+        <v>-58.40382</v>
       </c>
       <c r="N146" t="n">
-        <v>-34.578546</v>
+        <v>-34.594385</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P146" t="inlineStr">
@@ -12865,7 +12865,7 @@
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>ATH-B</t>
+          <t>AGU-A</t>
         </is>
       </c>
       <c r="R146" t="inlineStr">
@@ -12877,7 +12877,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t xml:space="preserve">10062 </t>
+          <t xml:space="preserve">10042 </t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -12887,7 +12887,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>HUMBOLDT 1556</t>
+          <t>PARAGUAY 5310</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -12930,10 +12930,10 @@
         <v>1</v>
       </c>
       <c r="M147" t="n">
-        <v>-58.436737</v>
+        <v>-58.43218</v>
       </c>
       <c r="N147" t="n">
-        <v>-34.58597</v>
+        <v>-34.578546</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -12947,7 +12947,7 @@
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>ATH-M</t>
+          <t>ATH-B</t>
         </is>
       </c>
       <c r="R147" t="inlineStr">
@@ -12959,7 +12959,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t xml:space="preserve">10066 </t>
+          <t xml:space="preserve">10062 </t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -12969,7 +12969,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARENALES 3640 </t>
+          <t>HUMBOLDT 1556</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -12990,12 +12990,12 @@
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr">
         <is>
-          <t>DESMONTAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
@@ -13012,10 +13012,10 @@
         <v>1</v>
       </c>
       <c r="M148" t="n">
-        <v>-58.413584</v>
+        <v>-58.436737</v>
       </c>
       <c r="N148" t="n">
-        <v>-34.58551</v>
+        <v>-34.58597</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -13029,7 +13029,7 @@
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>AGU-L</t>
+          <t>ATH-M</t>
         </is>
       </c>
       <c r="R148" t="inlineStr">
@@ -13041,7 +13041,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t xml:space="preserve">10067 </t>
+          <t xml:space="preserve">10066 </t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -13051,7 +13051,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>CHARCAS 3601</t>
+          <t xml:space="preserve">ARENALES 3640 </t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -13072,17 +13072,17 @@
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>DESMONTAR COLUMNA</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -13094,10 +13094,10 @@
         <v>1</v>
       </c>
       <c r="M149" t="n">
-        <v>-58.415912</v>
+        <v>-58.413584</v>
       </c>
       <c r="N149" t="n">
-        <v>-34.588977</v>
+        <v>-34.58551</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -13111,7 +13111,7 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>VCR-E</t>
+          <t>AGU-L</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">
@@ -13123,7 +13123,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t xml:space="preserve">10072 </t>
+          <t xml:space="preserve">10067 </t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -13133,7 +13133,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>SANTA FE AV. 3470</t>
+          <t>CHARCAS 3601</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -13164,7 +13164,7 @@
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
@@ -13176,10 +13176,10 @@
         <v>1</v>
       </c>
       <c r="M150" t="n">
-        <v>-58.413885</v>
+        <v>-58.415912</v>
       </c>
       <c r="N150" t="n">
-        <v>-34.586628</v>
+        <v>-34.588977</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -13193,7 +13193,7 @@
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>VCR-G</t>
+          <t>VCR-E</t>
         </is>
       </c>
       <c r="R150" t="inlineStr">
@@ -13205,7 +13205,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t xml:space="preserve">10080 </t>
+          <t xml:space="preserve">10072 </t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>THAMES 549</t>
+          <t>SANTA FE AV. 3470</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -13258,10 +13258,10 @@
         <v>1</v>
       </c>
       <c r="M151" t="n">
-        <v>-58.442534</v>
+        <v>-58.413885</v>
       </c>
       <c r="N151" t="n">
-        <v>-34.59499</v>
+        <v>-34.586628</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -13275,7 +13275,7 @@
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>VCR-G</t>
         </is>
       </c>
       <c r="R151" t="inlineStr">
@@ -13287,7 +13287,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t xml:space="preserve">10082 </t>
+          <t xml:space="preserve">10080 </t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -13297,7 +13297,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>TAGLE 2562</t>
+          <t>THAMES 549</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -13318,12 +13318,12 @@
       <c r="G152" t="inlineStr"/>
       <c r="H152" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
@@ -13340,14 +13340,14 @@
         <v>1</v>
       </c>
       <c r="M152" t="n">
-        <v>-58.400188</v>
+        <v>-58.442534</v>
       </c>
       <c r="N152" t="n">
-        <v>-34.583882</v>
+        <v>-34.59499</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P152" t="inlineStr">
@@ -13357,7 +13357,7 @@
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>AGU-I</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R152" t="inlineStr">
@@ -13369,7 +13369,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t xml:space="preserve">10083 </t>
+          <t xml:space="preserve">10082 </t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -13379,7 +13379,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>ORTIZ DE OCAMPO 2639</t>
+          <t>TAGLE 2562</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -13400,12 +13400,12 @@
       <c r="G153" t="inlineStr"/>
       <c r="H153" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
@@ -13422,10 +13422,10 @@
         <v>1</v>
       </c>
       <c r="M153" t="n">
-        <v>-58.404652</v>
+        <v>-58.400188</v>
       </c>
       <c r="N153" t="n">
-        <v>-34.58263</v>
+        <v>-34.583882</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -13439,7 +13439,7 @@
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>AGU-N</t>
+          <t>AGU-I</t>
         </is>
       </c>
       <c r="R153" t="inlineStr">
@@ -13451,7 +13451,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t xml:space="preserve">10098 </t>
+          <t xml:space="preserve">10083 </t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>DORREGO AV. 2635</t>
+          <t>ORTIZ DE OCAMPO 2639</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -13482,12 +13482,12 @@
       <c r="G154" t="inlineStr"/>
       <c r="H154" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
@@ -13504,14 +13504,14 @@
         <v>1</v>
       </c>
       <c r="M154" t="n">
-        <v>-58.433857</v>
+        <v>-58.404652</v>
       </c>
       <c r="N154" t="n">
-        <v>-34.57424</v>
+        <v>-34.58263</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P154" t="inlineStr">
@@ -13521,7 +13521,7 @@
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>BLO-G</t>
+          <t>AGU-N</t>
         </is>
       </c>
       <c r="R154" t="inlineStr">
@@ -13533,7 +13533,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t xml:space="preserve">10103 </t>
+          <t xml:space="preserve">10098 </t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -13543,7 +13543,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>DORREGO AV. 2765</t>
+          <t>DORREGO AV. 2635</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -13564,12 +13564,12 @@
       <c r="G155" t="inlineStr"/>
       <c r="H155" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
@@ -13586,10 +13586,10 @@
         <v>1</v>
       </c>
       <c r="M155" t="n">
-        <v>-58.432319</v>
+        <v>-58.433857</v>
       </c>
       <c r="N155" t="n">
-        <v>-34.574385</v>
+        <v>-34.57424</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -13615,7 +13615,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t xml:space="preserve">10104 </t>
+          <t xml:space="preserve">10103 </t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -13625,7 +13625,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t xml:space="preserve">DORREGO AV. 4050 </t>
+          <t>DORREGO AV. 2765</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -13646,12 +13646,12 @@
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAMBIAR COLUMNA </t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
@@ -13668,10 +13668,10 @@
         <v>1</v>
       </c>
       <c r="M156" t="n">
-        <v>-58.416882</v>
+        <v>-58.432319</v>
       </c>
       <c r="N156" t="n">
-        <v>-34.562655</v>
+        <v>-34.574385</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -13685,7 +13685,7 @@
       </c>
       <c r="Q156" t="inlineStr">
         <is>
-          <t>BLO-?</t>
+          <t>BLO-G</t>
         </is>
       </c>
       <c r="R156" t="inlineStr">
@@ -13697,7 +13697,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t xml:space="preserve">10131 </t>
+          <t xml:space="preserve">10104 </t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -13707,7 +13707,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t xml:space="preserve">PARAGUAY 4022 </t>
+          <t xml:space="preserve">DORREGO AV. 4050 </t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -13728,49 +13728,213 @@
       <c r="G157" t="inlineStr"/>
       <c r="H157" t="inlineStr">
         <is>
+          <t xml:space="preserve">CAMBIAR COLUMNA </t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L157" t="n">
+        <v>1</v>
+      </c>
+      <c r="M157" t="n">
+        <v>-58.416882</v>
+      </c>
+      <c r="N157" t="n">
+        <v>-34.562655</v>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t>BLO-?</t>
+        </is>
+      </c>
+      <c r="R157" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10129 </t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>5/14/2026</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>ALVAREZ, JULIAN 1890</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr"/>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>COLUMNA INCLINADA</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L158" t="n">
+        <v>1</v>
+      </c>
+      <c r="M158" t="n">
+        <v>-58.42056</v>
+      </c>
+      <c r="N158" t="n">
+        <v>-34.590217</v>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>VCR-D</t>
+        </is>
+      </c>
+      <c r="R158" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10131 </t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>5/14/2026</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PARAGUAY 4022 </t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr"/>
+      <c r="H159" t="inlineStr">
+        <is>
           <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
-      <c r="I157" t="inlineStr">
+      <c r="I159" t="inlineStr">
         <is>
           <t>Cambio</t>
         </is>
       </c>
-      <c r="J157" t="inlineStr">
+      <c r="J159" t="inlineStr">
         <is>
           <t>Nodo/Fuente Teco</t>
         </is>
       </c>
-      <c r="K157" t="inlineStr">
+      <c r="K159" t="inlineStr">
         <is>
           <t>Pasante</t>
         </is>
       </c>
-      <c r="L157" t="n">
-        <v>1</v>
-      </c>
-      <c r="M157" t="n">
+      <c r="L159" t="n">
+        <v>1</v>
+      </c>
+      <c r="M159" t="n">
         <v>-58.419652</v>
       </c>
-      <c r="N157" t="n">
+      <c r="N159" t="n">
         <v>-34.588271</v>
       </c>
-      <c r="O157" t="inlineStr">
+      <c r="O159" t="inlineStr">
         <is>
           <t>Palermo</t>
         </is>
       </c>
-      <c r="P157" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q157" t="inlineStr">
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q159" t="inlineStr">
         <is>
           <t>VCR-K</t>
         </is>
       </c>
-      <c r="R157" t="inlineStr">
+      <c r="R159" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-01 11:47:37)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_PEBCOM.xlsx
+++ b/mapa_interactivo_PEBCOM.xlsx
@@ -7655,7 +7655,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814105825</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -7913,7 +7913,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814107507</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -7999,7 +7999,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814107596</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -10405,7 +10405,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr"/>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>814108527</t>
+        </is>
+      </c>
       <c r="H117" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -10569,7 +10573,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr"/>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>814108607</t>
+        </is>
+      </c>
       <c r="H119" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -10651,7 +10659,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr"/>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>814108619</t>
+        </is>
+      </c>
       <c r="H120" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -10733,7 +10745,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>814108632</t>
+        </is>
+      </c>
       <c r="H121" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -10815,7 +10831,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr"/>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>814108642</t>
+        </is>
+      </c>
       <c r="H122" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -10897,7 +10917,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G123" t="inlineStr"/>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>814108650</t>
+        </is>
+      </c>
       <c r="H123" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA, POSIBLE NUEVA ALEDAÑA</t>
@@ -11061,7 +11085,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G125" t="inlineStr"/>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>814108660</t>
+        </is>
+      </c>
       <c r="H125" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -11143,7 +11171,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr"/>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>814109172</t>
+        </is>
+      </c>
       <c r="H126" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -11225,7 +11257,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr"/>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>814109219</t>
+        </is>
+      </c>
       <c r="H127" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -11717,7 +11753,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr"/>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>814108116</t>
+        </is>
+      </c>
       <c r="H133" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -11799,7 +11839,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G134" t="inlineStr"/>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>814108196</t>
+        </is>
+      </c>
       <c r="H134" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -12045,7 +12089,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G137" t="inlineStr"/>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>814108322</t>
+        </is>
+      </c>
       <c r="H137" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -12127,7 +12175,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G138" t="inlineStr"/>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>814108343</t>
+        </is>
+      </c>
       <c r="H138" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -12455,7 +12507,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G142" t="inlineStr"/>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>814108377</t>
+        </is>
+      </c>
       <c r="H142" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -12619,7 +12675,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G144" t="inlineStr"/>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>814108458</t>
+        </is>
+      </c>
       <c r="H144" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -12783,7 +12843,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G146" t="inlineStr"/>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>814108469</t>
+        </is>
+      </c>
       <c r="H146" t="inlineStr">
         <is>
           <t xml:space="preserve">CAMBIAR COLUMNA </t>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-01 13:05:35)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_PEBCOM.xlsx
+++ b/mapa_interactivo_PEBCOM.xlsx
@@ -11343,7 +11343,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G128" t="inlineStr"/>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>814109418</t>
+        </is>
+      </c>
       <c r="H128" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -11507,7 +11511,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G130" t="inlineStr"/>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>814109740</t>
+        </is>
+      </c>
       <c r="H130" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -11589,7 +11597,11 @@
           <t>PEBCOM</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr"/>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>814109788</t>
+        </is>
+      </c>
       <c r="H131" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-02 15:37:17)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_PEBCOM.xlsx
+++ b/mapa_interactivo_PEBCOM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R148"/>
+  <dimension ref="A1:R155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,17 +439,17 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Proveedor Asignado</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>OT</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -531,17 +531,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>ICD30334341</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>ICD30334341</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -613,17 +613,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>791764767</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>791764767</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -699,17 +699,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>798897149</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>798897149</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -781,17 +781,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>798897163</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>798897163</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -863,17 +863,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>798897384</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>798897384</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -945,17 +945,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>799246642</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>799246642</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1031,17 +1031,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>784675618</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>784675618</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -1113,17 +1113,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>799540497</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>799540497</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1199,17 +1199,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>784655947</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>784655947</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1285,17 +1285,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>803607889</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>803607889</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1371,17 +1371,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>803608480</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>803608480</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1457,17 +1457,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>803651203</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>803651203</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1543,17 +1543,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>803825124</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>803825124</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1629,17 +1629,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>804309752</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>804309752</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1715,17 +1715,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>804316147</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>804316147</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1801,17 +1801,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>804333522</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>804333522</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1887,17 +1887,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>804634219</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>804634219</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1973,17 +1973,17 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>804838861</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>804838861</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2059,17 +2059,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>805655369</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>805655369</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2145,17 +2145,17 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>ICD30592749</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>ICD30592749</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2231,17 +2231,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>805707245</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>805707245</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2317,17 +2317,17 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>805707264</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>805707264</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2403,17 +2403,17 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>805707278</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>805707278</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2489,17 +2489,17 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>805722772</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>805722772</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2575,17 +2575,17 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>806926557</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>806926557</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2661,17 +2661,17 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>806926806</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>806926806</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2747,17 +2747,17 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>806926927</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>806926927</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2833,17 +2833,17 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>807044071</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>807044071</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2919,17 +2919,17 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>807605730</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>807605730</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -3001,17 +3001,17 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>807762871</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>807762871</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3087,17 +3087,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>807971967</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>807971967</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3173,17 +3173,17 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808373635</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>808373635</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3259,17 +3259,17 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808430941</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>808430941</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -3345,17 +3345,17 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808460898</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>808460898</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -3431,17 +3431,17 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808460897</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>808460897</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3517,17 +3517,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808571975</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>808571975</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3603,17 +3603,17 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808571980</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>808571980</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3689,17 +3689,17 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808571985</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>808571985</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3775,17 +3775,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808733917</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>808733917</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3861,17 +3861,17 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808918705</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>808918705</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3947,17 +3947,17 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>809065854</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>809065854</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -4033,17 +4033,17 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>809526157</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>809526157</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -4119,17 +4119,17 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>809526162</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>809526162</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4205,17 +4205,17 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>809837500</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>809837500</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -4291,17 +4291,17 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810038995</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>810038995</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -4377,17 +4377,17 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>01095943</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>01095943</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -4463,17 +4463,17 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>ICD31463422</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>ICD31463422</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -4549,17 +4549,17 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810421921</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>810421921</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -4635,17 +4635,17 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
+          <t>01230434</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>01230434</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -4721,17 +4721,17 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>01450977</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>01450977</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -4807,17 +4807,17 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>01229656</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>01229656</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -4893,17 +4893,17 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t xml:space="preserve">01638326 </t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t xml:space="preserve">01638326 </t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -4979,17 +4979,17 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810853935</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>810853935</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -5065,17 +5065,17 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810877555</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>810877555</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -5151,17 +5151,17 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810877633</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>810877633</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -5237,17 +5237,17 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810984538</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>810984538</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -5323,17 +5323,17 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t xml:space="preserve">01749376 </t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t xml:space="preserve">01749376 </t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -5409,17 +5409,17 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811131649</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>811131649</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -5495,17 +5495,17 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -5581,17 +5581,17 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811198746</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>811198746</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -5667,17 +5667,17 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811198700</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>811198700</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -5753,17 +5753,17 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811198697</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>811198697</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -5839,17 +5839,17 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811238652</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>811238652</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -5925,17 +5925,17 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -6011,17 +6011,17 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811238686</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>811238686</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -6097,17 +6097,17 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t xml:space="preserve">02511365 </t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t xml:space="preserve">02511365 </t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -6183,17 +6183,17 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811454223</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>811454223</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -6269,17 +6269,17 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811454198</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>811454198</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -6355,17 +6355,17 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811454194</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>811454194</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -6441,17 +6441,17 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811454103</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>811454103</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -6527,17 +6527,17 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811453983</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>811453983</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -6613,17 +6613,17 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811453963</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>811453963</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -6699,17 +6699,17 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811454281</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>811454281</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -6785,17 +6785,17 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811498056</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>811498056</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -6871,17 +6871,17 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -6957,17 +6957,17 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811627110</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>811627110</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -7043,17 +7043,17 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811627090</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>811627090</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -7129,17 +7129,17 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -7215,17 +7215,17 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811627063</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>811627063</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -7301,17 +7301,17 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812440089</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>812440089</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -7387,17 +7387,17 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812440183</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>812440183</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -7473,17 +7473,17 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812440495</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>812440495</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -7559,17 +7559,17 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812440260</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>812440260</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -7645,17 +7645,17 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814105825</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>814105825</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -7731,17 +7731,17 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -7817,17 +7817,17 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -7903,17 +7903,17 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814107507</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>814107507</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -7989,17 +7989,17 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814107596</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>814107596</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -8075,17 +8075,17 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812879521</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>812879521</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -8161,17 +8161,17 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812879559</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>812879559</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -8247,17 +8247,17 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812879925</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>812879925</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -8333,17 +8333,17 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812880742</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>812880742</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -8419,17 +8419,17 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046389</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>813046389</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -8505,17 +8505,17 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046715</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>813046715</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -8591,17 +8591,17 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046718</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>813046718</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -8677,17 +8677,17 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046724</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>813046724</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -8763,17 +8763,17 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046778</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>813046778</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -8849,17 +8849,17 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813304793</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>813304793</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -8935,17 +8935,17 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813350523</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>813350523</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -9021,17 +9021,17 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813350536</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>813350536</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -9107,17 +9107,17 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813304889</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>813304889</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -9193,17 +9193,17 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813304917</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>813304917</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -9279,17 +9279,17 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813305004</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>813305004</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -9365,17 +9365,17 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813350615</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>813350615</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -9451,17 +9451,17 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813352568</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>813352568</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -9537,17 +9537,17 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813352603</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>813352603</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -9623,17 +9623,17 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813631416</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>813631416</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -9709,17 +9709,17 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813631417</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>813631417</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
@@ -9795,17 +9795,17 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813631425</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>813631425</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -9881,17 +9881,17 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813631432</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>813631432</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -9967,17 +9967,17 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813631446</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>813631446</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
@@ -10053,17 +10053,17 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813631449</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>813631449</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -10139,17 +10139,17 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813631451</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>813631451</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -10225,17 +10225,17 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813631452</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>813631452</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -10311,17 +10311,17 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813631921</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>813631921</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -10397,17 +10397,17 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108527</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>814108527</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -10483,15 +10483,19 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814111029</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G118" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
       <c r="H118" t="inlineStr">
         <is>
           <t>COLUMNA INCLINADA</t>
@@ -10499,7 +10503,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -10565,17 +10569,17 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108607</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>814108607</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -10651,17 +10655,17 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108619</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>814108619</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -10737,17 +10741,17 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108632</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>814108632</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -10823,17 +10827,17 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108642</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>814108642</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -10909,17 +10913,17 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108650</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>814108650</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -10993,17 +10997,17 @@
           <t>14</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G124" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
       <c r="H124" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -11077,17 +11081,17 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108660</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>814108660</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -11163,17 +11167,17 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814109172</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>814109172</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -11249,17 +11253,17 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814109219</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>814109219</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -11335,17 +11339,17 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814109418</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>814109418</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -11419,17 +11423,17 @@
           <t>14</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G129" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
       <c r="H129" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -11503,17 +11507,17 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814109740</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>814109740</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -11589,17 +11593,17 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814109788</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>814109788</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -11673,17 +11677,17 @@
           <t>14</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G132" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
       <c r="H132" t="inlineStr">
         <is>
           <t>COLUMNA INCLINADA</t>
@@ -11757,17 +11761,17 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108116</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>814108116</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -11843,17 +11847,17 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108196</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>814108196</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -11929,15 +11933,19 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814111706</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G135" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
       <c r="H135" t="inlineStr">
         <is>
           <t>COLUMNA INCLINADA</t>
@@ -11945,7 +11953,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -12009,17 +12017,17 @@
           <t>2</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G136" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
       <c r="H136" t="inlineStr">
         <is>
           <t>COLUMNA INCLINADA</t>
@@ -12093,17 +12101,17 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108322</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>814108322</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -12179,17 +12187,17 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108343</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>814108343</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -12263,17 +12271,17 @@
           <t>14</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G139" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
       <c r="H139" t="inlineStr">
         <is>
           <t>DESMONTAR COLUMNA</t>
@@ -12345,17 +12353,17 @@
           <t>14</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="E140" t="inlineStr"/>
       <c r="F140" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G140" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
       <c r="H140" t="inlineStr">
         <is>
           <t>COLUMNA INCLINADA</t>
@@ -12429,15 +12437,19 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814111751</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G141" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
       <c r="H141" t="inlineStr">
         <is>
           <t>COLUMNA INCLINADA</t>
@@ -12445,7 +12457,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
@@ -12511,17 +12523,17 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108377</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>814108377</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
@@ -12597,15 +12609,19 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814111784</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G143" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
       <c r="H143" t="inlineStr">
         <is>
           <t>COLUMNA INCLINADA</t>
@@ -12613,7 +12629,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
@@ -12679,17 +12695,17 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108458</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>814108458</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
@@ -12765,15 +12781,19 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814111791</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G145" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
       <c r="H145" t="inlineStr">
         <is>
           <t>COLUMNA INCLINADA</t>
@@ -12781,7 +12801,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
@@ -12847,17 +12867,17 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108469</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>814108469</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
@@ -12933,15 +12953,19 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814111804</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G147" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
       <c r="H147" t="inlineStr">
         <is>
           <t>COLUMNA INCLINADA</t>
@@ -12949,7 +12973,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
@@ -13013,17 +13037,17 @@
           <t>14</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="E148" t="inlineStr"/>
       <c r="F148" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G148" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
       <c r="H148" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -13069,6 +13093,608 @@
         </is>
       </c>
       <c r="R148" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>-775</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>11 DE SEPTIEMBRE DE 1888 996</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L149" t="n">
+        <v>1</v>
+      </c>
+      <c r="M149" t="n">
+        <v>-58.442098</v>
+      </c>
+      <c r="N149" t="n">
+        <v>-34.568762</v>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>BLO-G</t>
+        </is>
+      </c>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>-781</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>ARENALES 3658</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>814125568</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L150" t="n">
+        <v>1</v>
+      </c>
+      <c r="M150" t="n">
+        <v>-58.413717</v>
+      </c>
+      <c r="N150" t="n">
+        <v>-34.585425</v>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>AGU-L</t>
+        </is>
+      </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>-782</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>ARMENIA 1800</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>814125577</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L151" t="n">
+        <v>1</v>
+      </c>
+      <c r="M151" t="n">
+        <v>-58.426328</v>
+      </c>
+      <c r="N151" t="n">
+        <v>-34.588734</v>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>VCR-F</t>
+        </is>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>-787</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>CHENAUT, INDALESIO, GRAL. AV. 1945</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L152" t="n">
+        <v>1</v>
+      </c>
+      <c r="M152" t="n">
+        <v>-58.432822</v>
+      </c>
+      <c r="N152" t="n">
+        <v>-34.571917</v>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>BLO-H</t>
+        </is>
+      </c>
+      <c r="R152" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>-796</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>CABRERA, JOSE A. 4723</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>814125624</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L153" t="n">
+        <v>1</v>
+      </c>
+      <c r="M153" t="n">
+        <v>-58.429431</v>
+      </c>
+      <c r="N153" t="n">
+        <v>-34.591921</v>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>VCR-F</t>
+        </is>
+      </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>-797</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>CHARCAS 3248</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>814125633</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>columna chocada</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L154" t="n">
+        <v>1</v>
+      </c>
+      <c r="M154" t="n">
+        <v>-58.411747</v>
+      </c>
+      <c r="N154" t="n">
+        <v>-34.592175</v>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>AGU-C</t>
+        </is>
+      </c>
+      <c r="R154" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>-805</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>MATIENZO, BENJAMIN, TENIENTE 1510</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>814125656</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L155" t="n">
+        <v>1</v>
+      </c>
+      <c r="M155" t="n">
+        <v>-58.432345</v>
+      </c>
+      <c r="N155" t="n">
+        <v>-34.566345</v>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>BLO-I</t>
+        </is>
+      </c>
+      <c r="R155" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-03 11:57:52)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_PEBCOM.xlsx
+++ b/mapa_interactivo_PEBCOM.xlsx
@@ -5925,7 +5925,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>Pendiente ADM OT GxC</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -6861,7 +6861,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Beruti 3012</t>
+          <t>BERUTI 3012</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -6871,7 +6871,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>Pendiente ADM OT GxC</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -7129,7 +7129,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>Pendiente ADM OT GxC</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-08 12:33:41)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_PEBCOM.xlsx
+++ b/mapa_interactivo_PEBCOM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R153"/>
+  <dimension ref="A1:R152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9693,7 +9693,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>9080</t>
+          <t>9081</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -9703,7 +9703,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>LACROZE, FEDERICO AV. 2338</t>
+          <t>SOLDADO DE LA INDEPENDENCIA 1102</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -9718,7 +9718,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>813631432</t>
+          <t>813631446</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -9733,7 +9733,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
@@ -9750,24 +9750,24 @@
         <v>1</v>
       </c>
       <c r="M109" t="n">
-        <v>-58.444112</v>
+        <v>-58.438595</v>
       </c>
       <c r="N109" t="n">
-        <v>-34.569261</v>
+        <v>-34.565168</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>BLO-L</t>
+          <t>BLO-J</t>
         </is>
       </c>
       <c r="R109" t="inlineStr">
@@ -9779,7 +9779,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>9081</t>
+          <t>9083</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -9789,7 +9789,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>SOLDADO DE LA INDEPENDENCIA 1102</t>
+          <t>ARCE 949</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -9804,7 +9804,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>813631446</t>
+          <t>813631449</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -9819,7 +9819,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -9836,10 +9836,10 @@
         <v>1</v>
       </c>
       <c r="M110" t="n">
-        <v>-58.438595</v>
+        <v>-58.437217</v>
       </c>
       <c r="N110" t="n">
-        <v>-34.565168</v>
+        <v>-34.567174</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -9865,7 +9865,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>9083</t>
+          <t>9084</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -9875,7 +9875,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>ARCE 949</t>
+          <t xml:space="preserve">CAMPOS, LUIS M. AV. 1188 </t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -9890,7 +9890,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>813631449</t>
+          <t>813631451</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -9900,12 +9900,12 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -9922,10 +9922,10 @@
         <v>1</v>
       </c>
       <c r="M111" t="n">
-        <v>-58.437217</v>
+        <v>-58.44018</v>
       </c>
       <c r="N111" t="n">
-        <v>-34.567174</v>
+        <v>-34.565612</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -9939,7 +9939,7 @@
       </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t>BLO-J</t>
+          <t>BLO-L</t>
         </is>
       </c>
       <c r="R111" t="inlineStr">
@@ -9951,7 +9951,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>9084</t>
+          <t>9085</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -9961,7 +9961,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAMPOS, LUIS M. AV. 1188 </t>
+          <t>VILLANUEVA 1212</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -9976,7 +9976,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>813631451</t>
+          <t>813631452</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -9986,12 +9986,12 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -10008,19 +10008,19 @@
         <v>1</v>
       </c>
       <c r="M112" t="n">
-        <v>-58.44018</v>
+        <v>-58.441718</v>
       </c>
       <c r="N112" t="n">
-        <v>-34.565612</v>
+        <v>-34.566411</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q112" t="inlineStr">
@@ -10037,22 +10037,22 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>9085</t>
+          <t>S00477293</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>4/30/2026</t>
+          <t>5/10/2026</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>VILLANUEVA 1212</t>
+          <t xml:space="preserve"> ARENALES 2552</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -10062,7 +10062,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>813631452</t>
+          <t>813631921</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -10072,12 +10072,12 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
@@ -10094,24 +10094,24 @@
         <v>1</v>
       </c>
       <c r="M113" t="n">
-        <v>-58.441718</v>
+        <v>-58.402534</v>
       </c>
       <c r="N113" t="n">
-        <v>-34.566411</v>
+        <v>-34.593133</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>BLO-L</t>
+          <t>AGU-F</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
@@ -10123,17 +10123,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>S00477293</t>
+          <t>S01385955</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>5/10/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ARENALES 2552</t>
+          <t>POSADAS 1391</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -10148,7 +10148,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>813631921</t>
+          <t>814108527</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -10180,10 +10180,10 @@
         <v>1</v>
       </c>
       <c r="M114" t="n">
-        <v>-58.402534</v>
+        <v>-58.385947</v>
       </c>
       <c r="N114" t="n">
-        <v>-34.593133</v>
+        <v>-34.588156</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -10197,7 +10197,7 @@
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>AGU-F</t>
+          <t>RET-L</t>
         </is>
       </c>
       <c r="R114" t="inlineStr">
@@ -10209,7 +10209,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>S01385955</t>
+          <t>S00432540</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -10219,12 +10219,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>POSADAS 1391</t>
+          <t>DUMONT, SANTOS 2618</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -10234,7 +10234,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>814108527</t>
+          <t>814111029</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -10244,7 +10244,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -10266,14 +10266,14 @@
         <v>1</v>
       </c>
       <c r="M115" t="n">
-        <v>-58.385947</v>
+        <v>-58.440439</v>
       </c>
       <c r="N115" t="n">
-        <v>-34.588156</v>
+        <v>-34.575416</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P115" t="inlineStr">
@@ -10283,7 +10283,7 @@
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t>RET-L</t>
+          <t>COG-B</t>
         </is>
       </c>
       <c r="R115" t="inlineStr">
@@ -10295,7 +10295,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>S00432540</t>
+          <t xml:space="preserve">9179 </t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -10305,7 +10305,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>DUMONT, SANTOS 2618</t>
+          <t>ARAOZ 2289</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -10320,7 +10320,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>814111029</t>
+          <t>814108607</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -10330,7 +10330,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -10352,10 +10352,10 @@
         <v>1</v>
       </c>
       <c r="M116" t="n">
-        <v>-58.440439</v>
+        <v>-58.418131</v>
       </c>
       <c r="N116" t="n">
-        <v>-34.575416</v>
+        <v>-34.58774</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -10369,7 +10369,7 @@
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>COG-B</t>
+          <t>VCR-G</t>
         </is>
       </c>
       <c r="R116" t="inlineStr">
@@ -10381,7 +10381,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t xml:space="preserve">9179 </t>
+          <t xml:space="preserve">9180 </t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -10391,7 +10391,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ARAOZ 2289</t>
+          <t>MIGUELETES 1156</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -10406,7 +10406,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>814108607</t>
+          <t>814108619</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -10438,10 +10438,10 @@
         <v>1</v>
       </c>
       <c r="M117" t="n">
-        <v>-58.418131</v>
+        <v>-58.438274</v>
       </c>
       <c r="N117" t="n">
-        <v>-34.58774</v>
+        <v>-34.564049</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -10455,7 +10455,7 @@
       </c>
       <c r="Q117" t="inlineStr">
         <is>
-          <t>VCR-G</t>
+          <t>BLO-J</t>
         </is>
       </c>
       <c r="R117" t="inlineStr">
@@ -10467,7 +10467,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t xml:space="preserve">9180 </t>
+          <t xml:space="preserve">9115 </t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -10477,7 +10477,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>MIGUELETES 1156</t>
+          <t>NEWBERY, JORGE 1694</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -10492,7 +10492,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>814108619</t>
+          <t>814108632</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -10524,10 +10524,10 @@
         <v>1</v>
       </c>
       <c r="M118" t="n">
-        <v>-58.438274</v>
+        <v>-58.434721</v>
       </c>
       <c r="N118" t="n">
-        <v>-34.564049</v>
+        <v>-34.567241</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -10541,7 +10541,7 @@
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>BLO-J</t>
+          <t>BLO-H</t>
         </is>
       </c>
       <c r="R118" t="inlineStr">
@@ -10553,7 +10553,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t xml:space="preserve">9115 </t>
+          <t xml:space="preserve">9116 </t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -10563,7 +10563,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>NEWBERY, JORGE 1694</t>
+          <t>GOROSTIAGA 1514</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -10578,7 +10578,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>814108632</t>
+          <t>814108642</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -10610,10 +10610,10 @@
         <v>1</v>
       </c>
       <c r="M119" t="n">
-        <v>-58.434721</v>
+        <v>-58.435738</v>
       </c>
       <c r="N119" t="n">
-        <v>-34.567241</v>
+        <v>-34.564606</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -10627,7 +10627,7 @@
       </c>
       <c r="Q119" t="inlineStr">
         <is>
-          <t>BLO-H</t>
+          <t>BLO-J</t>
         </is>
       </c>
       <c r="R119" t="inlineStr">
@@ -10639,7 +10639,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t xml:space="preserve">9116 </t>
+          <t xml:space="preserve">9117 </t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -10649,7 +10649,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>GOROSTIAGA 1514</t>
+          <t>MAURE 1590</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>814108642</t>
+          <t>814108650</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -10674,7 +10674,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA, POSIBLE NUEVA ALEDAÑA</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -10696,10 +10696,10 @@
         <v>1</v>
       </c>
       <c r="M120" t="n">
-        <v>-58.435738</v>
+        <v>-58.435011</v>
       </c>
       <c r="N120" t="n">
-        <v>-34.564606</v>
+        <v>-34.56566</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -10725,7 +10725,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t xml:space="preserve">9117 </t>
+          <t xml:space="preserve">9118 </t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -10735,7 +10735,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>MAURE 1590</t>
+          <t>ORTEGA Y GASSET 1590</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -10748,11 +10748,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>814108650</t>
-        </is>
-      </c>
+      <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -10760,7 +10756,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA, POSIBLE NUEVA ALEDAÑA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -10770,7 +10766,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -10782,10 +10778,10 @@
         <v>1</v>
       </c>
       <c r="M121" t="n">
-        <v>-58.435011</v>
+        <v>-58.430774</v>
       </c>
       <c r="N121" t="n">
-        <v>-34.56566</v>
+        <v>-34.568179</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -10799,7 +10795,7 @@
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>BLO-J</t>
+          <t>BLO-I</t>
         </is>
       </c>
       <c r="R121" t="inlineStr">
@@ -10811,7 +10807,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t xml:space="preserve">9118 </t>
+          <t>9120</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -10821,7 +10817,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>ORTEGA Y GASSET 1590</t>
+          <t>ARCE 867</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -10834,7 +10830,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F122" t="inlineStr"/>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>814108660</t>
+        </is>
+      </c>
       <c r="G122" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -10852,7 +10852,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -10864,10 +10864,10 @@
         <v>1</v>
       </c>
       <c r="M122" t="n">
-        <v>-58.430774</v>
+        <v>-58.436255</v>
       </c>
       <c r="N122" t="n">
-        <v>-34.568179</v>
+        <v>-34.567733</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -10881,7 +10881,7 @@
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>BLO-I</t>
+          <t>BLO-J</t>
         </is>
       </c>
       <c r="R122" t="inlineStr">
@@ -10893,7 +10893,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>9120</t>
+          <t xml:space="preserve">9193 </t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -10903,7 +10903,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>ARCE 867</t>
+          <t>CRAMER 315</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -10918,7 +10918,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>814108660</t>
+          <t>814109172</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -10950,10 +10950,10 @@
         <v>1</v>
       </c>
       <c r="M123" t="n">
-        <v>-58.436255</v>
+        <v>-58.443403</v>
       </c>
       <c r="N123" t="n">
-        <v>-34.567733</v>
+        <v>-34.575666</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -10967,7 +10967,7 @@
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>BLO-J</t>
+          <t>ATH-B</t>
         </is>
       </c>
       <c r="R123" t="inlineStr">
@@ -10979,7 +10979,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t xml:space="preserve">9193 </t>
+          <t xml:space="preserve">9199 </t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -10989,7 +10989,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>CRAMER 315</t>
+          <t>ARMENIA 1553</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -11004,7 +11004,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>814109172</t>
+          <t>814109219</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -11036,10 +11036,10 @@
         <v>1</v>
       </c>
       <c r="M124" t="n">
-        <v>-58.443403</v>
+        <v>-58.428639</v>
       </c>
       <c r="N124" t="n">
-        <v>-34.575666</v>
+        <v>-34.59039</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -11053,7 +11053,7 @@
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>ATH-B</t>
+          <t>VCR-F</t>
         </is>
       </c>
       <c r="R124" t="inlineStr">
@@ -11065,7 +11065,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t xml:space="preserve">9199 </t>
+          <t>S00497843</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -11075,12 +11075,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>ARMENIA 1553</t>
+          <t>MANSILLA, LUCIO NORBERTO, GENERAL 2610</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -11090,7 +11090,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>814109219</t>
+          <t>814109418</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -11122,14 +11122,14 @@
         <v>1</v>
       </c>
       <c r="M125" t="n">
-        <v>-58.428639</v>
+        <v>-58.404726</v>
       </c>
       <c r="N125" t="n">
-        <v>-34.59039</v>
+        <v>-34.596069</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P125" t="inlineStr">
@@ -11139,7 +11139,7 @@
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>VCR-F</t>
+          <t>AGU-A</t>
         </is>
       </c>
       <c r="R125" t="inlineStr">
@@ -11151,7 +11151,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>S00497843</t>
+          <t>S00522384</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -11161,12 +11161,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>MANSILLA, LUCIO NORBERTO, GENERAL 2610</t>
+          <t>FRAY JUSTO SANTAMARIA DE ORO 2734</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -11174,11 +11174,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>814109418</t>
-        </is>
-      </c>
+      <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -11196,7 +11192,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -11208,14 +11204,14 @@
         <v>1</v>
       </c>
       <c r="M126" t="n">
-        <v>-58.404726</v>
+        <v>-58.422183</v>
       </c>
       <c r="N126" t="n">
-        <v>-34.596069</v>
+        <v>-34.576849</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
@@ -11225,7 +11221,7 @@
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>AGU-A</t>
+          <t>VCR-M</t>
         </is>
       </c>
       <c r="R126" t="inlineStr">
@@ -11237,7 +11233,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>S00522384</t>
+          <t xml:space="preserve">9220 </t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -11247,7 +11243,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>FRAY JUSTO SANTAMARIA DE ORO 2734</t>
+          <t>ARMENIA 1829</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -11260,7 +11256,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr"/>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>814109740</t>
+        </is>
+      </c>
       <c r="G127" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -11278,7 +11278,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -11290,10 +11290,10 @@
         <v>1</v>
       </c>
       <c r="M127" t="n">
-        <v>-58.422183</v>
+        <v>-58.425803</v>
       </c>
       <c r="N127" t="n">
-        <v>-34.576849</v>
+        <v>-34.588513</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -11307,7 +11307,7 @@
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>VCR-M</t>
+          <t>VCR-K</t>
         </is>
       </c>
       <c r="R127" t="inlineStr">
@@ -11319,7 +11319,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t xml:space="preserve">9220 </t>
+          <t xml:space="preserve">9945 </t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -11329,7 +11329,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>ARMENIA 1829</t>
+          <t>LACROZE, FEDERICO AV. 1938</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -11344,7 +11344,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>814109740</t>
+          <t>814109788</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -11376,10 +11376,10 @@
         <v>1</v>
       </c>
       <c r="M128" t="n">
-        <v>-58.425803</v>
+        <v>-58.440759</v>
       </c>
       <c r="N128" t="n">
-        <v>-34.588513</v>
+        <v>-34.565819</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -11393,7 +11393,7 @@
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>VCR-K</t>
+          <t>BLO-L</t>
         </is>
       </c>
       <c r="R128" t="inlineStr">
@@ -11405,17 +11405,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t xml:space="preserve">9945 </t>
+          <t xml:space="preserve">10033 </t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>LACROZE, FEDERICO AV. 1938</t>
+          <t>ESTADO DE PALESTINA 1192</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -11428,11 +11428,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr">
-        <is>
-          <t>814109788</t>
-        </is>
-      </c>
+      <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -11440,17 +11436,17 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -11462,10 +11458,10 @@
         <v>1</v>
       </c>
       <c r="M129" t="n">
-        <v>-58.440759</v>
+        <v>-58.424388</v>
       </c>
       <c r="N129" t="n">
-        <v>-34.565819</v>
+        <v>-34.59632</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -11479,7 +11475,7 @@
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>BLO-L</t>
+          <t>VCR-D</t>
         </is>
       </c>
       <c r="R129" t="inlineStr">
@@ -11491,7 +11487,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t xml:space="preserve">10033 </t>
+          <t xml:space="preserve">9157 </t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -11501,7 +11497,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ESTADO DE PALESTINA 1192</t>
+          <t>GUATEMALA 5078</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -11514,7 +11510,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F130" t="inlineStr"/>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>814108116</t>
+        </is>
+      </c>
       <c r="G130" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -11522,17 +11522,17 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -11544,10 +11544,10 @@
         <v>1</v>
       </c>
       <c r="M130" t="n">
-        <v>-58.424388</v>
+        <v>-58.427895</v>
       </c>
       <c r="N130" t="n">
-        <v>-34.59632</v>
+        <v>-34.583677</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -11561,7 +11561,7 @@
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>VCR-D</t>
+          <t>VCR-P</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
@@ -11573,7 +11573,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t xml:space="preserve">9157 </t>
+          <t xml:space="preserve">9924 </t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -11583,7 +11583,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>GUATEMALA 5078</t>
+          <t>CORDOBA AV. 4089</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -11598,7 +11598,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>814108116</t>
+          <t>814108196</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -11630,10 +11630,10 @@
         <v>1</v>
       </c>
       <c r="M131" t="n">
-        <v>-58.427895</v>
+        <v>-58.424553</v>
       </c>
       <c r="N131" t="n">
-        <v>-34.583677</v>
+        <v>-34.59709</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -11647,7 +11647,7 @@
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>VCR-P</t>
+          <t>VCR-D</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
@@ -11659,7 +11659,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t xml:space="preserve">9924 </t>
+          <t xml:space="preserve">10047 </t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -11669,7 +11669,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>CORDOBA AV. 4089</t>
+          <t>NEWBERY, JORGE 2410</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -11684,7 +11684,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>814108196</t>
+          <t>814111706</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
@@ -11694,7 +11694,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -11716,10 +11716,10 @@
         <v>1</v>
       </c>
       <c r="M132" t="n">
-        <v>-58.424553</v>
+        <v>-58.440973</v>
       </c>
       <c r="N132" t="n">
-        <v>-34.59709</v>
+        <v>-34.572415</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -11733,7 +11733,7 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>VCR-D</t>
+          <t>COG-B</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
@@ -11745,7 +11745,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">10047 </t>
+          <t>S01035299</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -11755,12 +11755,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>NEWBERY, JORGE 2410</t>
+          <t>ECUADOR 1390</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -11768,11 +11768,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F133" t="inlineStr">
-        <is>
-          <t>814111706</t>
-        </is>
-      </c>
+      <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -11785,12 +11781,12 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -11802,14 +11798,14 @@
         <v>1</v>
       </c>
       <c r="M133" t="n">
-        <v>-58.440973</v>
+        <v>-58.40382</v>
       </c>
       <c r="N133" t="n">
-        <v>-34.572415</v>
+        <v>-34.594385</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
@@ -11819,7 +11815,7 @@
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>COG-B</t>
+          <t>AGU-A</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
@@ -11831,7 +11827,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>S01035299</t>
+          <t xml:space="preserve">10042 </t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -11841,12 +11837,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ECUADOR 1390</t>
+          <t>PARAGUAY 5310</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -11854,7 +11850,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F134" t="inlineStr"/>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>814108322</t>
+        </is>
+      </c>
       <c r="G134" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -11862,17 +11862,17 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -11884,14 +11884,14 @@
         <v>1</v>
       </c>
       <c r="M134" t="n">
-        <v>-58.40382</v>
+        <v>-58.43218</v>
       </c>
       <c r="N134" t="n">
-        <v>-34.594385</v>
+        <v>-34.578546</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
@@ -11901,7 +11901,7 @@
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>AGU-A</t>
+          <t>ATH-B</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
@@ -11913,7 +11913,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">10042 </t>
+          <t xml:space="preserve">10062 </t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -11923,7 +11923,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>PARAGUAY 5310</t>
+          <t>HUMBOLDT 1556</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -11938,7 +11938,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>814108322</t>
+          <t>814108343</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -11970,10 +11970,10 @@
         <v>1</v>
       </c>
       <c r="M135" t="n">
-        <v>-58.43218</v>
+        <v>-58.436737</v>
       </c>
       <c r="N135" t="n">
-        <v>-34.578546</v>
+        <v>-34.58597</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -11987,7 +11987,7 @@
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>ATH-B</t>
+          <t>ATH-M</t>
         </is>
       </c>
       <c r="R135" t="inlineStr">
@@ -11999,7 +11999,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">10062 </t>
+          <t xml:space="preserve">10066 </t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -12009,7 +12009,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>HUMBOLDT 1556</t>
+          <t xml:space="preserve">ARENALES 3640 </t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -12022,11 +12022,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F136" t="inlineStr">
-        <is>
-          <t>814108343</t>
-        </is>
-      </c>
+      <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -12034,12 +12030,12 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>DESMONTAR COLUMNA</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -12056,10 +12052,10 @@
         <v>1</v>
       </c>
       <c r="M136" t="n">
-        <v>-58.436737</v>
+        <v>-58.413584</v>
       </c>
       <c r="N136" t="n">
-        <v>-34.58597</v>
+        <v>-34.58551</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -12073,7 +12069,7 @@
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>ATH-M</t>
+          <t>AGU-L</t>
         </is>
       </c>
       <c r="R136" t="inlineStr">
@@ -12085,7 +12081,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">10066 </t>
+          <t xml:space="preserve">10067 </t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -12095,7 +12091,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARENALES 3640 </t>
+          <t>CHARCAS 3601</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -12116,17 +12112,17 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>DESMONTAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -12138,10 +12134,10 @@
         <v>1</v>
       </c>
       <c r="M137" t="n">
-        <v>-58.413584</v>
+        <v>-58.415912</v>
       </c>
       <c r="N137" t="n">
-        <v>-34.58551</v>
+        <v>-34.588977</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -12155,7 +12151,7 @@
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>AGU-L</t>
+          <t>VCR-E</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
@@ -12167,7 +12163,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">10067 </t>
+          <t xml:space="preserve">10072 </t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -12177,7 +12173,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>CHARCAS 3601</t>
+          <t>SANTA FE AV. 3470</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -12190,7 +12186,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F138" t="inlineStr"/>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>814111751</t>
+        </is>
+      </c>
       <c r="G138" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -12203,12 +12203,12 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -12220,10 +12220,10 @@
         <v>1</v>
       </c>
       <c r="M138" t="n">
-        <v>-58.415912</v>
+        <v>-58.413885</v>
       </c>
       <c r="N138" t="n">
-        <v>-34.588977</v>
+        <v>-34.586628</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -12237,7 +12237,7 @@
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>VCR-E</t>
+          <t>VCR-G</t>
         </is>
       </c>
       <c r="R138" t="inlineStr">
@@ -12249,7 +12249,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">10072 </t>
+          <t xml:space="preserve">10082 </t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -12259,7 +12259,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>SANTA FE AV. 3470</t>
+          <t>TAGLE 2562</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -12274,7 +12274,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>814111751</t>
+          <t>814108377</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -12284,7 +12284,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -12306,14 +12306,14 @@
         <v>1</v>
       </c>
       <c r="M139" t="n">
-        <v>-58.413885</v>
+        <v>-58.400188</v>
       </c>
       <c r="N139" t="n">
-        <v>-34.586628</v>
+        <v>-34.583882</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
@@ -12323,7 +12323,7 @@
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>VCR-G</t>
+          <t>AGU-I</t>
         </is>
       </c>
       <c r="R139" t="inlineStr">
@@ -12335,7 +12335,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">10082 </t>
+          <t xml:space="preserve">10083 </t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -12345,7 +12345,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>TAGLE 2562</t>
+          <t>ORTIZ DE OCAMPO 2639</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -12360,7 +12360,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>814108377</t>
+          <t>814111784</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
@@ -12370,7 +12370,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -12392,10 +12392,10 @@
         <v>1</v>
       </c>
       <c r="M140" t="n">
-        <v>-58.400188</v>
+        <v>-58.404652</v>
       </c>
       <c r="N140" t="n">
-        <v>-34.583882</v>
+        <v>-34.58263</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -12409,7 +12409,7 @@
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>AGU-I</t>
+          <t>AGU-N</t>
         </is>
       </c>
       <c r="R140" t="inlineStr">
@@ -12421,7 +12421,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">10083 </t>
+          <t xml:space="preserve">10098 </t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -12431,7 +12431,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>ORTIZ DE OCAMPO 2639</t>
+          <t>DORREGO AV. 2635</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -12446,7 +12446,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>814111784</t>
+          <t>814108458</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -12456,7 +12456,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -12478,14 +12478,14 @@
         <v>1</v>
       </c>
       <c r="M141" t="n">
-        <v>-58.404652</v>
+        <v>-58.433857</v>
       </c>
       <c r="N141" t="n">
-        <v>-34.58263</v>
+        <v>-34.57424</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P141" t="inlineStr">
@@ -12495,7 +12495,7 @@
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>AGU-N</t>
+          <t>BLO-G</t>
         </is>
       </c>
       <c r="R141" t="inlineStr">
@@ -12507,7 +12507,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">10098 </t>
+          <t xml:space="preserve">10103 </t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -12517,7 +12517,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>DORREGO AV. 2635</t>
+          <t>DORREGO AV. 2765</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -12532,7 +12532,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>814108458</t>
+          <t>814111791</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
@@ -12542,7 +12542,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -12564,10 +12564,10 @@
         <v>1</v>
       </c>
       <c r="M142" t="n">
-        <v>-58.433857</v>
+        <v>-58.432319</v>
       </c>
       <c r="N142" t="n">
-        <v>-34.57424</v>
+        <v>-34.574385</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -12593,7 +12593,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">10103 </t>
+          <t xml:space="preserve">10104 </t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -12603,7 +12603,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>DORREGO AV. 2765</t>
+          <t xml:space="preserve">DORREGO AV. 4050 </t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -12618,7 +12618,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>814111791</t>
+          <t>814108469</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
@@ -12628,7 +12628,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t xml:space="preserve">CAMBIAR COLUMNA </t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -12650,10 +12650,10 @@
         <v>1</v>
       </c>
       <c r="M143" t="n">
-        <v>-58.432319</v>
+        <v>-58.416882</v>
       </c>
       <c r="N143" t="n">
-        <v>-34.574385</v>
+        <v>-34.562655</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -12667,7 +12667,7 @@
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>BLO-G</t>
+          <t>BLO-?</t>
         </is>
       </c>
       <c r="R143" t="inlineStr">
@@ -12679,7 +12679,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">10104 </t>
+          <t xml:space="preserve">10129 </t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -12689,7 +12689,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t xml:space="preserve">DORREGO AV. 4050 </t>
+          <t>ALVAREZ, JULIAN 1890</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -12704,7 +12704,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>814108469</t>
+          <t>814111804</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
@@ -12714,7 +12714,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAMBIAR COLUMNA </t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -12729,17 +12729,17 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L144" t="n">
         <v>1</v>
       </c>
       <c r="M144" t="n">
-        <v>-58.416882</v>
+        <v>-58.42056</v>
       </c>
       <c r="N144" t="n">
-        <v>-34.562655</v>
+        <v>-34.590217</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -12753,7 +12753,7 @@
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>BLO-?</t>
+          <t>VCR-D</t>
         </is>
       </c>
       <c r="R144" t="inlineStr">
@@ -12765,7 +12765,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">10129 </t>
+          <t xml:space="preserve">10131 </t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -12775,7 +12775,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>ALVAREZ, JULIAN 1890</t>
+          <t xml:space="preserve">PARAGUAY 4022 </t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -12788,11 +12788,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F145" t="inlineStr">
-        <is>
-          <t>814111804</t>
-        </is>
-      </c>
+      <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -12800,7 +12796,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -12810,22 +12806,22 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L145" t="n">
         <v>1</v>
       </c>
       <c r="M145" t="n">
-        <v>-58.42056</v>
+        <v>-58.419652</v>
       </c>
       <c r="N145" t="n">
-        <v>-34.590217</v>
+        <v>-34.588271</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -12839,7 +12835,7 @@
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>VCR-D</t>
+          <t>VCR-K</t>
         </is>
       </c>
       <c r="R145" t="inlineStr">
@@ -12851,17 +12847,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">10131 </t>
+          <t>-775</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>6/2/2026</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t xml:space="preserve">PARAGUAY 4022 </t>
+          <t>11 DE SEPTIEMBRE DE 1888 996</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -12874,7 +12870,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F146" t="inlineStr"/>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
       <c r="G146" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -12882,7 +12882,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -12892,7 +12892,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -12904,10 +12904,10 @@
         <v>1</v>
       </c>
       <c r="M146" t="n">
-        <v>-58.419652</v>
+        <v>-58.442098</v>
       </c>
       <c r="N146" t="n">
-        <v>-34.588271</v>
+        <v>-34.568762</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>VCR-K</t>
+          <t>BLO-G</t>
         </is>
       </c>
       <c r="R146" t="inlineStr">
@@ -12933,7 +12933,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>-775</t>
+          <t>-781</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -12943,7 +12943,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>11 DE SEPTIEMBRE DE 1888 996</t>
+          <t>ARENALES 3658</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -12958,7 +12958,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814125568</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -12978,7 +12978,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -12990,10 +12990,10 @@
         <v>1</v>
       </c>
       <c r="M147" t="n">
-        <v>-58.442098</v>
+        <v>-58.413717</v>
       </c>
       <c r="N147" t="n">
-        <v>-34.568762</v>
+        <v>-34.585425</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -13007,7 +13007,7 @@
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>BLO-G</t>
+          <t>AGU-L</t>
         </is>
       </c>
       <c r="R147" t="inlineStr">
@@ -13019,7 +13019,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>-781</t>
+          <t>-782</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -13029,7 +13029,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>ARENALES 3658</t>
+          <t>ARMENIA 1800</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -13044,7 +13044,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>814125568</t>
+          <t>814125577</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -13076,10 +13076,10 @@
         <v>1</v>
       </c>
       <c r="M148" t="n">
-        <v>-58.413717</v>
+        <v>-58.426328</v>
       </c>
       <c r="N148" t="n">
-        <v>-34.585425</v>
+        <v>-34.588734</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -13093,7 +13093,7 @@
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>AGU-L</t>
+          <t>VCR-F</t>
         </is>
       </c>
       <c r="R148" t="inlineStr">
@@ -13105,7 +13105,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>-782</t>
+          <t>-787</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -13115,7 +13115,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>ARMENIA 1800</t>
+          <t>CHENAUT, INDALESIO, GRAL. AV. 1945</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -13130,7 +13130,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>814125577</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -13150,7 +13150,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -13162,10 +13162,10 @@
         <v>1</v>
       </c>
       <c r="M149" t="n">
-        <v>-58.426328</v>
+        <v>-58.432822</v>
       </c>
       <c r="N149" t="n">
-        <v>-34.588734</v>
+        <v>-34.571917</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -13179,7 +13179,7 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>VCR-F</t>
+          <t>BLO-H</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">
@@ -13191,7 +13191,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>-787</t>
+          <t>-796</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -13201,7 +13201,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>CHENAUT, INDALESIO, GRAL. AV. 1945</t>
+          <t>CABRERA, JOSE A. 4723</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -13216,7 +13216,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814125624</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -13236,7 +13236,7 @@
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
@@ -13248,10 +13248,10 @@
         <v>1</v>
       </c>
       <c r="M150" t="n">
-        <v>-58.432822</v>
+        <v>-58.429431</v>
       </c>
       <c r="N150" t="n">
-        <v>-34.571917</v>
+        <v>-34.591921</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -13265,7 +13265,7 @@
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>BLO-H</t>
+          <t>VCR-F</t>
         </is>
       </c>
       <c r="R150" t="inlineStr">
@@ -13277,7 +13277,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>-796</t>
+          <t>-797</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -13287,12 +13287,12 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>CABRERA, JOSE A. 4723</t>
+          <t>CHARCAS 3248</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -13302,7 +13302,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>814125624</t>
+          <t>814125633</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -13312,7 +13312,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>columna chocada</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -13334,14 +13334,14 @@
         <v>1</v>
       </c>
       <c r="M151" t="n">
-        <v>-58.429431</v>
+        <v>-58.411747</v>
       </c>
       <c r="N151" t="n">
-        <v>-34.591921</v>
+        <v>-34.592175</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P151" t="inlineStr">
@@ -13351,7 +13351,7 @@
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>VCR-F</t>
+          <t>AGU-C</t>
         </is>
       </c>
       <c r="R151" t="inlineStr">
@@ -13363,7 +13363,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>-797</t>
+          <t>-805</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -13373,12 +13373,12 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>CHARCAS 3248</t>
+          <t>MATIENZO, BENJAMIN, TENIENTE 1510</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -13388,7 +13388,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>814125633</t>
+          <t>814125656</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -13398,7 +13398,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>columna chocada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -13420,14 +13420,14 @@
         <v>1</v>
       </c>
       <c r="M152" t="n">
-        <v>-58.411747</v>
+        <v>-58.432345</v>
       </c>
       <c r="N152" t="n">
-        <v>-34.592175</v>
+        <v>-34.566345</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P152" t="inlineStr">
@@ -13437,96 +13437,10 @@
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>AGU-C</t>
+          <t>BLO-I</t>
         </is>
       </c>
       <c r="R152" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>-805</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>6/2/2026</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>MATIENZO, BENJAMIN, TENIENTE 1510</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="E153" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F153" t="inlineStr">
-        <is>
-          <t>814125656</t>
-        </is>
-      </c>
-      <c r="G153" t="inlineStr">
-        <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="H153" t="inlineStr">
-        <is>
-          <t>base corroida</t>
-        </is>
-      </c>
-      <c r="I153" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J153" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K153" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L153" t="n">
-        <v>1</v>
-      </c>
-      <c r="M153" t="n">
-        <v>-58.432345</v>
-      </c>
-      <c r="N153" t="n">
-        <v>-34.566345</v>
-      </c>
-      <c r="O153" t="inlineStr">
-        <is>
-          <t>Palermo</t>
-        </is>
-      </c>
-      <c r="P153" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q153" t="inlineStr">
-        <is>
-          <t>BLO-I</t>
-        </is>
-      </c>
-      <c r="R153" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-11 16:05:07)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_PEBCOM.xlsx
+++ b/mapa_interactivo_PEBCOM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R152"/>
+  <dimension ref="A1:R154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13446,6 +13446,178 @@
         </is>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>814446819</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>6/11/2026</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>ANGEL GALLARDO 946</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>814446819</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L153" t="n">
+        <v>0</v>
+      </c>
+      <c r="M153" t="n">
+        <v>-58.443588</v>
+      </c>
+      <c r="N153" t="n">
+        <v>-34.606863</v>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>ALM-O</t>
+        </is>
+      </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>814446825</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>6/11/2026</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>ANGEL GALLARDO 1084</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>814446825</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>PEBCOM</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L154" t="n">
+        <v>0</v>
+      </c>
+      <c r="M154" t="n">
+        <v>-58.445084</v>
+      </c>
+      <c r="N154" t="n">
+        <v>-34.60725</v>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>ALM-O</t>
+        </is>
+      </c>
+      <c r="R154" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-19 14:53:48)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_PEBCOM.xlsx
+++ b/mapa_interactivo_PEBCOM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R154"/>
+  <dimension ref="A1:R153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7973,17 +7973,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>8609</t>
+          <t>00781500</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>3/13/2026</t>
+          <t>3/21/2026</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>SEGUI JUAN FRANCISCO 4691</t>
+          <t>RAVIGNANI EMILIO DR 1498</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -7998,7 +7998,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>812879559</t>
+          <t>812879925</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -8008,7 +8008,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Cambiar Columna</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -8030,10 +8030,10 @@
         <v>1</v>
       </c>
       <c r="M89" t="n">
-        <v>-58.422229</v>
+        <v>-58.441411</v>
       </c>
       <c r="N89" t="n">
-        <v>-34.573148</v>
+        <v>-34.583443</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
@@ -8047,7 +8047,7 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>VCR-M</t>
+          <t>ATH-M</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
@@ -8059,22 +8059,22 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>00781500</t>
+          <t>8702</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>3/21/2026</t>
+          <t>3/28/2026</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>RAVIGNANI EMILIO DR 1498</t>
+          <t>JUNCAL 2249</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -8084,7 +8084,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>812879925</t>
+          <t>812880742</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -8116,14 +8116,14 @@
         <v>1</v>
       </c>
       <c r="M90" t="n">
-        <v>-58.441411</v>
+        <v>-58.399319</v>
       </c>
       <c r="N90" t="n">
-        <v>-34.583443</v>
+        <v>-34.592221</v>
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P90" t="inlineStr">
@@ -8133,34 +8133,34 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>ATH-M</t>
+          <t>RET-E</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.1RET</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>8702</t>
+          <t>8746</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>3/28/2026</t>
+          <t>4/7/2026</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>JUNCAL 2249</t>
+          <t>PARAGUAY 4237</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -8170,7 +8170,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>812880742</t>
+          <t>813046389</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -8190,7 +8190,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -8202,14 +8202,14 @@
         <v>1</v>
       </c>
       <c r="M91" t="n">
-        <v>-58.399319</v>
+        <v>-58.421616</v>
       </c>
       <c r="N91" t="n">
-        <v>-34.592221</v>
+        <v>-34.586608</v>
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P91" t="inlineStr">
@@ -8219,29 +8219,29 @@
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>RET-E</t>
+          <t>VCR-O</t>
         </is>
       </c>
       <c r="R91" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.1RET</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>8746</t>
+          <t>S00289486</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>4/7/2026</t>
+          <t>4/11/2026</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>PARAGUAY 4237</t>
+          <t>PARAGUAY 4585</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -8256,7 +8256,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>813046389</t>
+          <t>813046715</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -8276,7 +8276,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -8288,10 +8288,10 @@
         <v>1</v>
       </c>
       <c r="M92" t="n">
-        <v>-58.421616</v>
+        <v>-58.42498</v>
       </c>
       <c r="N92" t="n">
-        <v>-34.586608</v>
+        <v>-34.584031</v>
       </c>
       <c r="O92" t="inlineStr">
         <is>
@@ -8305,7 +8305,7 @@
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>VCR-O</t>
+          <t>VCR-P</t>
         </is>
       </c>
       <c r="R92" t="inlineStr">
@@ -8317,7 +8317,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>S00289486</t>
+          <t>S00325208</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -8327,7 +8327,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>PARAGUAY 4585</t>
+          <t>PARAGUAY 3711</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -8342,7 +8342,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>813046715</t>
+          <t>813046718</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -8374,10 +8374,10 @@
         <v>1</v>
       </c>
       <c r="M93" t="n">
-        <v>-58.42498</v>
+        <v>-58.416117</v>
       </c>
       <c r="N93" t="n">
-        <v>-34.584031</v>
+        <v>-34.590942</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
@@ -8391,7 +8391,7 @@
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>VCR-P</t>
+          <t>VCR-C</t>
         </is>
       </c>
       <c r="R93" t="inlineStr">
@@ -8403,7 +8403,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>S00325208</t>
+          <t>S00337251</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -8413,12 +8413,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>PARAGUAY 3711</t>
+          <t>SANCHEZ DE BUSTAMANTE 2450</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -8428,7 +8428,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>813046718</t>
+          <t>813046724</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -8460,14 +8460,14 @@
         <v>1</v>
       </c>
       <c r="M94" t="n">
-        <v>-58.416117</v>
+        <v>-58.403295</v>
       </c>
       <c r="N94" t="n">
-        <v>-34.590942</v>
+        <v>-34.585041</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P94" t="inlineStr">
@@ -8477,7 +8477,7 @@
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>VCR-C</t>
+          <t>AGU-H</t>
         </is>
       </c>
       <c r="R94" t="inlineStr">
@@ -8489,7 +8489,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>S00337251</t>
+          <t>S00364886</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -8499,12 +8499,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>SANCHEZ DE BUSTAMANTE 2450</t>
+          <t>MATIENZO BENJAMIN TENIENTE 1830</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>813046724</t>
+          <t>813046778</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -8546,14 +8546,14 @@
         <v>1</v>
       </c>
       <c r="M95" t="n">
-        <v>-58.403295</v>
+        <v>-58.434778</v>
       </c>
       <c r="N95" t="n">
-        <v>-34.585041</v>
+        <v>-34.569188</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P95" t="inlineStr">
@@ -8563,7 +8563,7 @@
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>AGU-H</t>
+          <t>BLO-I</t>
         </is>
       </c>
       <c r="R95" t="inlineStr">
@@ -8575,17 +8575,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>S00364886</t>
+          <t>PJ00009</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>4/11/2026</t>
+          <t>4/20/2026</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>MATIENZO BENJAMIN TENIENTE 1830</t>
+          <t>THAMES 1516</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -8600,7 +8600,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>813046778</t>
+          <t>813304793</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -8632,10 +8632,10 @@
         <v>1</v>
       </c>
       <c r="M96" t="n">
-        <v>-58.434778</v>
+        <v>-58.431966</v>
       </c>
       <c r="N96" t="n">
-        <v>-34.569188</v>
+        <v>-34.588553</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -8649,7 +8649,7 @@
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>BLO-I</t>
+          <t>VCR-F</t>
         </is>
       </c>
       <c r="R96" t="inlineStr">
@@ -8661,22 +8661,22 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>PJ00009</t>
+          <t>LR00001</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>4/20/2026</t>
+          <t>4/27/2026</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>THAMES 1516</t>
+          <t>BILLINGHURST 1796</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -8686,7 +8686,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>813304793</t>
+          <t>813350523</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -8718,14 +8718,14 @@
         <v>1</v>
       </c>
       <c r="M97" t="n">
-        <v>-58.431966</v>
+        <v>-58.409695</v>
       </c>
       <c r="N97" t="n">
-        <v>-34.588553</v>
+        <v>-34.589662</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P97" t="inlineStr">
@@ -8735,7 +8735,7 @@
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>VCR-F</t>
+          <t>AGU-D</t>
         </is>
       </c>
       <c r="R97" t="inlineStr">
@@ -8747,22 +8747,22 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>LR00001</t>
+          <t>PJ00040</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>4/27/2026</t>
+          <t>4/20/2026</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>BILLINGHURST 1796</t>
+          <t>HONDURAS 4822</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>813350523</t>
+          <t>813350536</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -8804,14 +8804,14 @@
         <v>1</v>
       </c>
       <c r="M98" t="n">
-        <v>-58.409695</v>
+        <v>-58.428528</v>
       </c>
       <c r="N98" t="n">
-        <v>-34.589662</v>
+        <v>-34.589872</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P98" t="inlineStr">
@@ -8821,7 +8821,7 @@
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>AGU-D</t>
+          <t>VCR-F</t>
         </is>
       </c>
       <c r="R98" t="inlineStr">
@@ -8833,7 +8833,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>PJ00040</t>
+          <t>AF00001</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -8843,7 +8843,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>HONDURAS 4822</t>
+          <t>SALGUERO, JERONIMO 1995</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -8858,7 +8858,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>813350536</t>
+          <t>813304889</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -8873,7 +8873,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -8890,10 +8890,10 @@
         <v>1</v>
       </c>
       <c r="M99" t="n">
-        <v>-58.428528</v>
+        <v>-58.413378</v>
       </c>
       <c r="N99" t="n">
-        <v>-34.589872</v>
+        <v>-34.587254</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -8907,7 +8907,7 @@
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>VCR-F</t>
+          <t>VCR-G</t>
         </is>
       </c>
       <c r="R99" t="inlineStr">
@@ -8919,7 +8919,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>AF00001</t>
+          <t>9006</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -8929,12 +8929,12 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>SALGUERO, JERONIMO 1995</t>
+          <t>CHARCAS 3250</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -8944,7 +8944,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>813304889</t>
+          <t>813304917</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -8976,14 +8976,14 @@
         <v>1</v>
       </c>
       <c r="M100" t="n">
-        <v>-58.413378</v>
+        <v>-58.41175</v>
       </c>
       <c r="N100" t="n">
-        <v>-34.587254</v>
+        <v>-34.592173</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P100" t="inlineStr">
@@ -8993,7 +8993,7 @@
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>VCR-G</t>
+          <t>AGU-C</t>
         </is>
       </c>
       <c r="R100" t="inlineStr">
@@ -9005,7 +9005,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>9006</t>
+          <t>8921</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -9015,12 +9015,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>CHARCAS 3250</t>
+          <t>DORREGO AV.2752</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>813304917</t>
+          <t>813305004</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -9062,14 +9062,14 @@
         <v>1</v>
       </c>
       <c r="M101" t="n">
-        <v>-58.41175</v>
+        <v>-58.43266</v>
       </c>
       <c r="N101" t="n">
-        <v>-34.592173</v>
+        <v>-34.574202</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P101" t="inlineStr">
@@ -9079,7 +9079,7 @@
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>AGU-C</t>
+          <t>BLO-G</t>
         </is>
       </c>
       <c r="R101" t="inlineStr">
@@ -9091,7 +9091,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>8921</t>
+          <t>S00419298</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -9101,12 +9101,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>DORREGO AV.2752</t>
+          <t>AUSTRIA 2354</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -9116,7 +9116,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>813305004</t>
+          <t>813350615</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -9148,14 +9148,14 @@
         <v>1</v>
       </c>
       <c r="M102" t="n">
-        <v>-58.43266</v>
+        <v>-58.401523</v>
       </c>
       <c r="N102" t="n">
-        <v>-34.574202</v>
+        <v>-34.586182</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
@@ -9165,7 +9165,7 @@
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>BLO-G</t>
+          <t>AGU-H</t>
         </is>
       </c>
       <c r="R102" t="inlineStr">
@@ -9177,22 +9177,22 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>S00419298</t>
+          <t>000025</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>4/20/2026</t>
+          <t>4/23/2026</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>AUSTRIA 2354</t>
+          <t>AV DORREGO 3900</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -9202,7 +9202,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>813350615</t>
+          <t>813352568</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -9212,7 +9212,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>POSTE CAIDO, VER POSIBILIDAD DE DESMONTE</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -9227,21 +9227,21 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L103" t="n">
         <v>1</v>
       </c>
       <c r="M103" t="n">
-        <v>-58.401523</v>
+        <v>-58.418801</v>
       </c>
       <c r="N103" t="n">
-        <v>-34.586182</v>
+        <v>-34.564182</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
@@ -9251,7 +9251,7 @@
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>AGU-H</t>
+          <t>BLO-?</t>
         </is>
       </c>
       <c r="R103" t="inlineStr">
@@ -9263,17 +9263,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>000025</t>
+          <t>9025</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>4/23/2026</t>
+          <t>4/24/2026</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>AV DORREGO 3900</t>
+          <t>ALVAREZ, JULIAN 2552</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -9288,7 +9288,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>813352568</t>
+          <t>813352603</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -9298,7 +9298,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>POSTE CAIDO, VER POSIBILIDAD DE DESMONTE</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -9313,17 +9313,17 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L104" t="n">
         <v>1</v>
       </c>
       <c r="M104" t="n">
-        <v>-58.418801</v>
+        <v>-58.413555</v>
       </c>
       <c r="N104" t="n">
-        <v>-34.564182</v>
+        <v>-34.585955</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
@@ -9337,7 +9337,7 @@
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>BLO-?</t>
+          <t>AGU-L</t>
         </is>
       </c>
       <c r="R104" t="inlineStr">
@@ -9349,17 +9349,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>9025</t>
+          <t>9062</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>4/24/2026</t>
+          <t>4/30/2026</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ALVAREZ, JULIAN 2552</t>
+          <t>BULNES 2550</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -9374,7 +9374,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>813352603</t>
+          <t>813631416</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -9384,12 +9384,12 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -9406,10 +9406,10 @@
         <v>1</v>
       </c>
       <c r="M105" t="n">
-        <v>-58.413555</v>
+        <v>-58.407013</v>
       </c>
       <c r="N105" t="n">
-        <v>-34.585955</v>
+        <v>-34.582645</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
@@ -9423,7 +9423,7 @@
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>AGU-L</t>
+          <t>AGU-N</t>
         </is>
       </c>
       <c r="R105" t="inlineStr">
@@ -9435,7 +9435,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>9062</t>
+          <t>9063</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -9445,7 +9445,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>BULNES 2550</t>
+          <t>DEL LIBERTADOR AV. 2030</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>813631416</t>
+          <t>813631417</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -9492,14 +9492,14 @@
         <v>1</v>
       </c>
       <c r="M106" t="n">
-        <v>-58.407013</v>
+        <v>-58.401882</v>
       </c>
       <c r="N106" t="n">
-        <v>-34.582645</v>
+        <v>-34.582006</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
@@ -9509,7 +9509,7 @@
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>AGU-N</t>
+          <t>AGU-I</t>
         </is>
       </c>
       <c r="R106" t="inlineStr">
@@ -9521,7 +9521,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>9063</t>
+          <t>9050</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -9531,7 +9531,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>DEL LIBERTADOR AV. 2030</t>
+          <t>CASTEX 3439</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -9546,7 +9546,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>813631417</t>
+          <t>813631425</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -9556,12 +9556,12 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -9578,14 +9578,14 @@
         <v>1</v>
       </c>
       <c r="M107" t="n">
-        <v>-58.401882</v>
+        <v>-58.406414</v>
       </c>
       <c r="N107" t="n">
-        <v>-34.582006</v>
+        <v>-34.577519</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
@@ -9595,7 +9595,7 @@
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>AGU-I</t>
+          <t>AGU-R</t>
         </is>
       </c>
       <c r="R107" t="inlineStr">
@@ -9607,7 +9607,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>9050</t>
+          <t>9081</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -9617,7 +9617,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>CASTEX 3439</t>
+          <t>SOLDADO DE LA INDEPENDENCIA 1102</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -9632,7 +9632,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>813631425</t>
+          <t>813631446</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -9642,7 +9642,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -9664,10 +9664,10 @@
         <v>1</v>
       </c>
       <c r="M108" t="n">
-        <v>-58.406414</v>
+        <v>-58.438595</v>
       </c>
       <c r="N108" t="n">
-        <v>-34.577519</v>
+        <v>-34.565168</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -9681,7 +9681,7 @@
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>AGU-R</t>
+          <t>BLO-J</t>
         </is>
       </c>
       <c r="R108" t="inlineStr">
@@ -9693,7 +9693,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>9081</t>
+          <t>9083</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -9703,7 +9703,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>SOLDADO DE LA INDEPENDENCIA 1102</t>
+          <t>ARCE 949</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -9718,7 +9718,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>813631446</t>
+          <t>813631449</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -9733,7 +9733,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
@@ -9750,10 +9750,10 @@
         <v>1</v>
       </c>
       <c r="M109" t="n">
-        <v>-58.438595</v>
+        <v>-58.437217</v>
       </c>
       <c r="N109" t="n">
-        <v>-34.565168</v>
+        <v>-34.567174</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -9779,7 +9779,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>9083</t>
+          <t>9084</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -9789,7 +9789,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>ARCE 949</t>
+          <t xml:space="preserve">CAMPOS, LUIS M. AV. 1188 </t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -9804,7 +9804,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>813631449</t>
+          <t>813631451</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -9814,12 +9814,12 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -9836,10 +9836,10 @@
         <v>1</v>
       </c>
       <c r="M110" t="n">
-        <v>-58.437217</v>
+        <v>-58.44018</v>
       </c>
       <c r="N110" t="n">
-        <v>-34.567174</v>
+        <v>-34.565612</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -9853,7 +9853,7 @@
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>BLO-J</t>
+          <t>BLO-L</t>
         </is>
       </c>
       <c r="R110" t="inlineStr">
@@ -9865,7 +9865,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>9084</t>
+          <t>9085</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -9875,7 +9875,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAMPOS, LUIS M. AV. 1188 </t>
+          <t>VILLANUEVA 1212</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -9890,7 +9890,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>813631451</t>
+          <t>813631452</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -9900,12 +9900,12 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -9922,19 +9922,19 @@
         <v>1</v>
       </c>
       <c r="M111" t="n">
-        <v>-58.44018</v>
+        <v>-58.441718</v>
       </c>
       <c r="N111" t="n">
-        <v>-34.565612</v>
+        <v>-34.566411</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q111" t="inlineStr">
@@ -9951,22 +9951,22 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>9085</t>
+          <t>S00477293</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>4/30/2026</t>
+          <t>5/10/2026</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>VILLANUEVA 1212</t>
+          <t xml:space="preserve"> ARENALES 2552</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -9976,7 +9976,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>813631452</t>
+          <t>813631921</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -9986,12 +9986,12 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -10008,24 +10008,24 @@
         <v>1</v>
       </c>
       <c r="M112" t="n">
-        <v>-58.441718</v>
+        <v>-58.402534</v>
       </c>
       <c r="N112" t="n">
-        <v>-34.566411</v>
+        <v>-34.593133</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>BLO-L</t>
+          <t>AGU-F</t>
         </is>
       </c>
       <c r="R112" t="inlineStr">
@@ -10037,17 +10037,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>S00477293</t>
+          <t>S01385955</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>5/10/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ARENALES 2552</t>
+          <t>POSADAS 1391</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -10062,7 +10062,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>813631921</t>
+          <t>814108527</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -10094,10 +10094,10 @@
         <v>1</v>
       </c>
       <c r="M113" t="n">
-        <v>-58.402534</v>
+        <v>-58.385947</v>
       </c>
       <c r="N113" t="n">
-        <v>-34.593133</v>
+        <v>-34.588156</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -10111,7 +10111,7 @@
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>AGU-F</t>
+          <t>RET-L</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
@@ -10123,7 +10123,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>S01385955</t>
+          <t>S00432540</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -10133,12 +10133,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>POSADAS 1391</t>
+          <t>DUMONT, SANTOS 2618</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -10148,7 +10148,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>814108527</t>
+          <t>814111029</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -10158,7 +10158,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -10180,14 +10180,14 @@
         <v>1</v>
       </c>
       <c r="M114" t="n">
-        <v>-58.385947</v>
+        <v>-58.440439</v>
       </c>
       <c r="N114" t="n">
-        <v>-34.588156</v>
+        <v>-34.575416</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P114" t="inlineStr">
@@ -10197,7 +10197,7 @@
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>RET-L</t>
+          <t>COG-B</t>
         </is>
       </c>
       <c r="R114" t="inlineStr">
@@ -10209,7 +10209,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>S00432540</t>
+          <t xml:space="preserve">9179 </t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -10219,7 +10219,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>DUMONT, SANTOS 2618</t>
+          <t>ARAOZ 2289</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -10234,7 +10234,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>814111029</t>
+          <t>814108607</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -10244,7 +10244,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -10266,10 +10266,10 @@
         <v>1</v>
       </c>
       <c r="M115" t="n">
-        <v>-58.440439</v>
+        <v>-58.418131</v>
       </c>
       <c r="N115" t="n">
-        <v>-34.575416</v>
+        <v>-34.58774</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -10283,7 +10283,7 @@
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t>COG-B</t>
+          <t>VCR-G</t>
         </is>
       </c>
       <c r="R115" t="inlineStr">
@@ -10295,7 +10295,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t xml:space="preserve">9179 </t>
+          <t xml:space="preserve">9180 </t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -10305,7 +10305,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>ARAOZ 2289</t>
+          <t>MIGUELETES 1156</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -10320,7 +10320,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>814108607</t>
+          <t>814108619</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -10352,10 +10352,10 @@
         <v>1</v>
       </c>
       <c r="M116" t="n">
-        <v>-58.418131</v>
+        <v>-58.438274</v>
       </c>
       <c r="N116" t="n">
-        <v>-34.58774</v>
+        <v>-34.564049</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -10369,7 +10369,7 @@
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>VCR-G</t>
+          <t>BLO-J</t>
         </is>
       </c>
       <c r="R116" t="inlineStr">
@@ -10381,7 +10381,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t xml:space="preserve">9180 </t>
+          <t xml:space="preserve">9115 </t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -10391,7 +10391,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>MIGUELETES 1156</t>
+          <t>NEWBERY, JORGE 1694</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -10406,7 +10406,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>814108619</t>
+          <t>814108632</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -10438,10 +10438,10 @@
         <v>1</v>
       </c>
       <c r="M117" t="n">
-        <v>-58.438274</v>
+        <v>-58.434721</v>
       </c>
       <c r="N117" t="n">
-        <v>-34.564049</v>
+        <v>-34.567241</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -10455,7 +10455,7 @@
       </c>
       <c r="Q117" t="inlineStr">
         <is>
-          <t>BLO-J</t>
+          <t>BLO-H</t>
         </is>
       </c>
       <c r="R117" t="inlineStr">
@@ -10467,7 +10467,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t xml:space="preserve">9115 </t>
+          <t xml:space="preserve">9116 </t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -10477,7 +10477,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>NEWBERY, JORGE 1694</t>
+          <t>GOROSTIAGA 1514</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -10492,7 +10492,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>814108632</t>
+          <t>814108642</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -10524,10 +10524,10 @@
         <v>1</v>
       </c>
       <c r="M118" t="n">
-        <v>-58.434721</v>
+        <v>-58.435738</v>
       </c>
       <c r="N118" t="n">
-        <v>-34.567241</v>
+        <v>-34.564606</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -10541,7 +10541,7 @@
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>BLO-H</t>
+          <t>BLO-J</t>
         </is>
       </c>
       <c r="R118" t="inlineStr">
@@ -10553,7 +10553,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t xml:space="preserve">9116 </t>
+          <t xml:space="preserve">9117 </t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -10563,7 +10563,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>GOROSTIAGA 1514</t>
+          <t>MAURE 1590</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -10578,7 +10578,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>814108642</t>
+          <t>814108650</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -10588,7 +10588,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA, POSIBLE NUEVA ALEDAÑA</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -10610,10 +10610,10 @@
         <v>1</v>
       </c>
       <c r="M119" t="n">
-        <v>-58.435738</v>
+        <v>-58.435011</v>
       </c>
       <c r="N119" t="n">
-        <v>-34.564606</v>
+        <v>-34.56566</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -10639,7 +10639,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t xml:space="preserve">9117 </t>
+          <t xml:space="preserve">9118 </t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -10649,7 +10649,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>MAURE 1590</t>
+          <t>ORTEGA Y GASSET 1590</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -10662,11 +10662,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>814108650</t>
-        </is>
-      </c>
+      <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -10674,7 +10670,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA, POSIBLE NUEVA ALEDAÑA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -10684,7 +10680,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -10696,10 +10692,10 @@
         <v>1</v>
       </c>
       <c r="M120" t="n">
-        <v>-58.435011</v>
+        <v>-58.430774</v>
       </c>
       <c r="N120" t="n">
-        <v>-34.56566</v>
+        <v>-34.568179</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -10713,7 +10709,7 @@
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>BLO-J</t>
+          <t>BLO-I</t>
         </is>
       </c>
       <c r="R120" t="inlineStr">
@@ -10725,7 +10721,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t xml:space="preserve">9118 </t>
+          <t>9120</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -10735,7 +10731,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ORTEGA Y GASSET 1590</t>
+          <t>ARCE 867</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -10748,7 +10744,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F121" t="inlineStr"/>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>814108660</t>
+        </is>
+      </c>
       <c r="G121" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -10766,7 +10766,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -10778,10 +10778,10 @@
         <v>1</v>
       </c>
       <c r="M121" t="n">
-        <v>-58.430774</v>
+        <v>-58.436255</v>
       </c>
       <c r="N121" t="n">
-        <v>-34.568179</v>
+        <v>-34.567733</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -10795,7 +10795,7 @@
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>BLO-I</t>
+          <t>BLO-J</t>
         </is>
       </c>
       <c r="R121" t="inlineStr">
@@ -10807,7 +10807,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>9120</t>
+          <t xml:space="preserve">9193 </t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -10817,7 +10817,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>ARCE 867</t>
+          <t>CRAMER 315</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -10832,7 +10832,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>814108660</t>
+          <t>814109172</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -10864,10 +10864,10 @@
         <v>1</v>
       </c>
       <c r="M122" t="n">
-        <v>-58.436255</v>
+        <v>-58.443403</v>
       </c>
       <c r="N122" t="n">
-        <v>-34.567733</v>
+        <v>-34.575666</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -10881,7 +10881,7 @@
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>BLO-J</t>
+          <t>ATH-B</t>
         </is>
       </c>
       <c r="R122" t="inlineStr">
@@ -10893,7 +10893,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t xml:space="preserve">9193 </t>
+          <t xml:space="preserve">9199 </t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -10903,7 +10903,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>CRAMER 315</t>
+          <t>ARMENIA 1553</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -10918,7 +10918,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>814109172</t>
+          <t>814109219</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -10950,10 +10950,10 @@
         <v>1</v>
       </c>
       <c r="M123" t="n">
-        <v>-58.443403</v>
+        <v>-58.428639</v>
       </c>
       <c r="N123" t="n">
-        <v>-34.575666</v>
+        <v>-34.59039</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -10967,7 +10967,7 @@
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>ATH-B</t>
+          <t>VCR-F</t>
         </is>
       </c>
       <c r="R123" t="inlineStr">
@@ -10979,7 +10979,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t xml:space="preserve">9199 </t>
+          <t>S00497843</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -10989,12 +10989,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>ARMENIA 1553</t>
+          <t>MANSILLA, LUCIO NORBERTO, GENERAL 2610</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -11004,7 +11004,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>814109219</t>
+          <t>814109418</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -11036,14 +11036,14 @@
         <v>1</v>
       </c>
       <c r="M124" t="n">
-        <v>-58.428639</v>
+        <v>-58.404726</v>
       </c>
       <c r="N124" t="n">
-        <v>-34.59039</v>
+        <v>-34.596069</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P124" t="inlineStr">
@@ -11053,7 +11053,7 @@
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>VCR-F</t>
+          <t>AGU-A</t>
         </is>
       </c>
       <c r="R124" t="inlineStr">
@@ -11065,7 +11065,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>S00497843</t>
+          <t>S00522384</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -11075,12 +11075,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>MANSILLA, LUCIO NORBERTO, GENERAL 2610</t>
+          <t>FRAY JUSTO SANTAMARIA DE ORO 2734</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -11088,11 +11088,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>814109418</t>
-        </is>
-      </c>
+      <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -11110,7 +11106,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -11122,14 +11118,14 @@
         <v>1</v>
       </c>
       <c r="M125" t="n">
-        <v>-58.404726</v>
+        <v>-58.422183</v>
       </c>
       <c r="N125" t="n">
-        <v>-34.596069</v>
+        <v>-34.576849</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P125" t="inlineStr">
@@ -11139,7 +11135,7 @@
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>AGU-A</t>
+          <t>VCR-M</t>
         </is>
       </c>
       <c r="R125" t="inlineStr">
@@ -11151,7 +11147,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>S00522384</t>
+          <t xml:space="preserve">9220 </t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -11161,7 +11157,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>FRAY JUSTO SANTAMARIA DE ORO 2734</t>
+          <t>ARMENIA 1829</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -11174,7 +11170,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F126" t="inlineStr"/>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>814109740</t>
+        </is>
+      </c>
       <c r="G126" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -11192,7 +11192,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -11204,10 +11204,10 @@
         <v>1</v>
       </c>
       <c r="M126" t="n">
-        <v>-58.422183</v>
+        <v>-58.425803</v>
       </c>
       <c r="N126" t="n">
-        <v>-34.576849</v>
+        <v>-34.588513</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -11221,7 +11221,7 @@
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>VCR-M</t>
+          <t>VCR-K</t>
         </is>
       </c>
       <c r="R126" t="inlineStr">
@@ -11233,7 +11233,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t xml:space="preserve">9220 </t>
+          <t xml:space="preserve">9945 </t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -11243,7 +11243,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>ARMENIA 1829</t>
+          <t>LACROZE, FEDERICO AV. 1938</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -11258,7 +11258,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>814109740</t>
+          <t>814109788</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -11290,10 +11290,10 @@
         <v>1</v>
       </c>
       <c r="M127" t="n">
-        <v>-58.425803</v>
+        <v>-58.440759</v>
       </c>
       <c r="N127" t="n">
-        <v>-34.588513</v>
+        <v>-34.565819</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -11307,7 +11307,7 @@
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>VCR-K</t>
+          <t>BLO-L</t>
         </is>
       </c>
       <c r="R127" t="inlineStr">
@@ -11319,17 +11319,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t xml:space="preserve">9945 </t>
+          <t xml:space="preserve">10033 </t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>LACROZE, FEDERICO AV. 1938</t>
+          <t>ESTADO DE PALESTINA 1192</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -11342,11 +11342,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>814109788</t>
-        </is>
-      </c>
+      <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -11354,17 +11350,17 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -11376,10 +11372,10 @@
         <v>1</v>
       </c>
       <c r="M128" t="n">
-        <v>-58.440759</v>
+        <v>-58.424388</v>
       </c>
       <c r="N128" t="n">
-        <v>-34.565819</v>
+        <v>-34.59632</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -11393,7 +11389,7 @@
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>BLO-L</t>
+          <t>VCR-D</t>
         </is>
       </c>
       <c r="R128" t="inlineStr">
@@ -11405,7 +11401,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t xml:space="preserve">10033 </t>
+          <t xml:space="preserve">9157 </t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -11415,7 +11411,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>ESTADO DE PALESTINA 1192</t>
+          <t>GUATEMALA 5078</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -11428,7 +11424,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr"/>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>814108116</t>
+        </is>
+      </c>
       <c r="G129" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -11436,17 +11436,17 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -11458,10 +11458,10 @@
         <v>1</v>
       </c>
       <c r="M129" t="n">
-        <v>-58.424388</v>
+        <v>-58.427895</v>
       </c>
       <c r="N129" t="n">
-        <v>-34.59632</v>
+        <v>-34.583677</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -11475,7 +11475,7 @@
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>VCR-D</t>
+          <t>VCR-P</t>
         </is>
       </c>
       <c r="R129" t="inlineStr">
@@ -11487,7 +11487,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t xml:space="preserve">9157 </t>
+          <t xml:space="preserve">9924 </t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -11497,7 +11497,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>GUATEMALA 5078</t>
+          <t>CORDOBA AV. 4089</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -11512,7 +11512,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>814108116</t>
+          <t>814108196</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -11544,10 +11544,10 @@
         <v>1</v>
       </c>
       <c r="M130" t="n">
-        <v>-58.427895</v>
+        <v>-58.424553</v>
       </c>
       <c r="N130" t="n">
-        <v>-34.583677</v>
+        <v>-34.59709</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -11561,7 +11561,7 @@
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>VCR-P</t>
+          <t>VCR-D</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
@@ -11573,7 +11573,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t xml:space="preserve">9924 </t>
+          <t xml:space="preserve">10047 </t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -11583,7 +11583,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>CORDOBA AV. 4089</t>
+          <t>NEWBERY, JORGE 2410</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -11598,7 +11598,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>814108196</t>
+          <t>814111706</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -11608,7 +11608,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -11630,10 +11630,10 @@
         <v>1</v>
       </c>
       <c r="M131" t="n">
-        <v>-58.424553</v>
+        <v>-58.440973</v>
       </c>
       <c r="N131" t="n">
-        <v>-34.59709</v>
+        <v>-34.572415</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -11647,7 +11647,7 @@
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>VCR-D</t>
+          <t>COG-B</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
@@ -11659,7 +11659,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t xml:space="preserve">10047 </t>
+          <t>S01035299</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -11669,12 +11669,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>NEWBERY, JORGE 2410</t>
+          <t>ECUADOR 1390</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -11682,11 +11682,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F132" t="inlineStr">
-        <is>
-          <t>814111706</t>
-        </is>
-      </c>
+      <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -11699,12 +11695,12 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -11716,14 +11712,14 @@
         <v>1</v>
       </c>
       <c r="M132" t="n">
-        <v>-58.440973</v>
+        <v>-58.40382</v>
       </c>
       <c r="N132" t="n">
-        <v>-34.572415</v>
+        <v>-34.594385</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P132" t="inlineStr">
@@ -11733,7 +11729,7 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>COG-B</t>
+          <t>AGU-A</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
@@ -11745,7 +11741,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>S01035299</t>
+          <t xml:space="preserve">10042 </t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -11755,12 +11751,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>ECUADOR 1390</t>
+          <t>PARAGUAY 5310</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -11768,7 +11764,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F133" t="inlineStr"/>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>814108322</t>
+        </is>
+      </c>
       <c r="G133" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -11776,17 +11776,17 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -11798,14 +11798,14 @@
         <v>1</v>
       </c>
       <c r="M133" t="n">
-        <v>-58.40382</v>
+        <v>-58.43218</v>
       </c>
       <c r="N133" t="n">
-        <v>-34.594385</v>
+        <v>-34.578546</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
@@ -11815,7 +11815,7 @@
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>AGU-A</t>
+          <t>ATH-B</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
@@ -11827,7 +11827,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">10042 </t>
+          <t xml:space="preserve">10062 </t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -11837,7 +11837,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>PARAGUAY 5310</t>
+          <t>HUMBOLDT 1556</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -11852,7 +11852,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>814108322</t>
+          <t>814108343</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
@@ -11884,10 +11884,10 @@
         <v>1</v>
       </c>
       <c r="M134" t="n">
-        <v>-58.43218</v>
+        <v>-58.436737</v>
       </c>
       <c r="N134" t="n">
-        <v>-34.578546</v>
+        <v>-34.58597</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -11901,7 +11901,7 @@
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>ATH-B</t>
+          <t>ATH-M</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
@@ -11913,7 +11913,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">10062 </t>
+          <t xml:space="preserve">10066 </t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -11923,7 +11923,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>HUMBOLDT 1556</t>
+          <t xml:space="preserve">ARENALES 3640 </t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -11936,11 +11936,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F135" t="inlineStr">
-        <is>
-          <t>814108343</t>
-        </is>
-      </c>
+      <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -11948,12 +11944,12 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>DESMONTAR COLUMNA</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -11970,10 +11966,10 @@
         <v>1</v>
       </c>
       <c r="M135" t="n">
-        <v>-58.436737</v>
+        <v>-58.413584</v>
       </c>
       <c r="N135" t="n">
-        <v>-34.58597</v>
+        <v>-34.58551</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -11987,7 +11983,7 @@
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>ATH-M</t>
+          <t>AGU-L</t>
         </is>
       </c>
       <c r="R135" t="inlineStr">
@@ -11999,7 +11995,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">10066 </t>
+          <t xml:space="preserve">10067 </t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -12009,7 +12005,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARENALES 3640 </t>
+          <t>CHARCAS 3601</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -12030,17 +12026,17 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>DESMONTAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -12052,10 +12048,10 @@
         <v>1</v>
       </c>
       <c r="M136" t="n">
-        <v>-58.413584</v>
+        <v>-58.415912</v>
       </c>
       <c r="N136" t="n">
-        <v>-34.58551</v>
+        <v>-34.588977</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -12069,7 +12065,7 @@
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>AGU-L</t>
+          <t>VCR-E</t>
         </is>
       </c>
       <c r="R136" t="inlineStr">
@@ -12081,7 +12077,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">10067 </t>
+          <t xml:space="preserve">10072 </t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -12091,7 +12087,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>CHARCAS 3601</t>
+          <t>SANTA FE AV. 3470</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -12104,7 +12100,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F137" t="inlineStr"/>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>814111751</t>
+        </is>
+      </c>
       <c r="G137" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -12117,12 +12117,12 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -12134,10 +12134,10 @@
         <v>1</v>
       </c>
       <c r="M137" t="n">
-        <v>-58.415912</v>
+        <v>-58.413885</v>
       </c>
       <c r="N137" t="n">
-        <v>-34.588977</v>
+        <v>-34.586628</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -12151,7 +12151,7 @@
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>VCR-E</t>
+          <t>VCR-G</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
@@ -12163,7 +12163,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">10072 </t>
+          <t xml:space="preserve">10082 </t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -12173,7 +12173,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>SANTA FE AV. 3470</t>
+          <t>TAGLE 2562</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -12188,7 +12188,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>814111751</t>
+          <t>814108377</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
@@ -12198,7 +12198,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -12220,14 +12220,14 @@
         <v>1</v>
       </c>
       <c r="M138" t="n">
-        <v>-58.413885</v>
+        <v>-58.400188</v>
       </c>
       <c r="N138" t="n">
-        <v>-34.586628</v>
+        <v>-34.583882</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P138" t="inlineStr">
@@ -12237,7 +12237,7 @@
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>VCR-G</t>
+          <t>AGU-I</t>
         </is>
       </c>
       <c r="R138" t="inlineStr">
@@ -12249,7 +12249,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">10082 </t>
+          <t xml:space="preserve">10083 </t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -12259,7 +12259,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>TAGLE 2562</t>
+          <t>ORTIZ DE OCAMPO 2639</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -12274,7 +12274,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>814108377</t>
+          <t>814111784</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -12284,7 +12284,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -12306,10 +12306,10 @@
         <v>1</v>
       </c>
       <c r="M139" t="n">
-        <v>-58.400188</v>
+        <v>-58.404652</v>
       </c>
       <c r="N139" t="n">
-        <v>-34.583882</v>
+        <v>-34.58263</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -12323,7 +12323,7 @@
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>AGU-I</t>
+          <t>AGU-N</t>
         </is>
       </c>
       <c r="R139" t="inlineStr">
@@ -12335,7 +12335,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">10083 </t>
+          <t xml:space="preserve">10098 </t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -12345,7 +12345,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>ORTIZ DE OCAMPO 2639</t>
+          <t>DORREGO AV. 2635</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -12360,7 +12360,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>814111784</t>
+          <t>814108458</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
@@ -12370,7 +12370,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -12392,14 +12392,14 @@
         <v>1</v>
       </c>
       <c r="M140" t="n">
-        <v>-58.404652</v>
+        <v>-58.433857</v>
       </c>
       <c r="N140" t="n">
-        <v>-34.58263</v>
+        <v>-34.57424</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P140" t="inlineStr">
@@ -12409,7 +12409,7 @@
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>AGU-N</t>
+          <t>BLO-G</t>
         </is>
       </c>
       <c r="R140" t="inlineStr">
@@ -12421,7 +12421,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">10098 </t>
+          <t xml:space="preserve">10103 </t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -12431,7 +12431,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>DORREGO AV. 2635</t>
+          <t>DORREGO AV. 2765</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -12446,7 +12446,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>814108458</t>
+          <t>814111791</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -12456,7 +12456,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -12478,10 +12478,10 @@
         <v>1</v>
       </c>
       <c r="M141" t="n">
-        <v>-58.433857</v>
+        <v>-58.432319</v>
       </c>
       <c r="N141" t="n">
-        <v>-34.57424</v>
+        <v>-34.574385</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -12507,7 +12507,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">10103 </t>
+          <t xml:space="preserve">10104 </t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -12517,7 +12517,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>DORREGO AV. 2765</t>
+          <t xml:space="preserve">DORREGO AV. 4050 </t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -12532,7 +12532,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>814111791</t>
+          <t>814108469</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
@@ -12542,7 +12542,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t xml:space="preserve">CAMBIAR COLUMNA </t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -12564,10 +12564,10 @@
         <v>1</v>
       </c>
       <c r="M142" t="n">
-        <v>-58.432319</v>
+        <v>-58.416882</v>
       </c>
       <c r="N142" t="n">
-        <v>-34.574385</v>
+        <v>-34.562655</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -12581,7 +12581,7 @@
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>BLO-G</t>
+          <t>BLO-?</t>
         </is>
       </c>
       <c r="R142" t="inlineStr">
@@ -12593,7 +12593,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">10104 </t>
+          <t xml:space="preserve">10129 </t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -12603,7 +12603,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t xml:space="preserve">DORREGO AV. 4050 </t>
+          <t>ALVAREZ, JULIAN 1890</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -12618,7 +12618,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>814108469</t>
+          <t>814111804</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
@@ -12628,7 +12628,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAMBIAR COLUMNA </t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -12643,17 +12643,17 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L143" t="n">
         <v>1</v>
       </c>
       <c r="M143" t="n">
-        <v>-58.416882</v>
+        <v>-58.42056</v>
       </c>
       <c r="N143" t="n">
-        <v>-34.562655</v>
+        <v>-34.590217</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -12667,7 +12667,7 @@
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>BLO-?</t>
+          <t>VCR-D</t>
         </is>
       </c>
       <c r="R143" t="inlineStr">
@@ -12679,7 +12679,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">10129 </t>
+          <t xml:space="preserve">10131 </t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -12689,7 +12689,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>ALVAREZ, JULIAN 1890</t>
+          <t xml:space="preserve">PARAGUAY 4022 </t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -12702,11 +12702,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F144" t="inlineStr">
-        <is>
-          <t>814111804</t>
-        </is>
-      </c>
+      <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -12714,7 +12710,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -12724,22 +12720,22 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L144" t="n">
         <v>1</v>
       </c>
       <c r="M144" t="n">
-        <v>-58.42056</v>
+        <v>-58.419652</v>
       </c>
       <c r="N144" t="n">
-        <v>-34.590217</v>
+        <v>-34.588271</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -12753,7 +12749,7 @@
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>VCR-D</t>
+          <t>VCR-K</t>
         </is>
       </c>
       <c r="R144" t="inlineStr">
@@ -12765,17 +12761,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">10131 </t>
+          <t>-775</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>6/2/2026</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t xml:space="preserve">PARAGUAY 4022 </t>
+          <t>11 DE SEPTIEMBRE DE 1888 996</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -12788,7 +12784,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F145" t="inlineStr"/>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
       <c r="G145" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -12796,7 +12796,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -12818,10 +12818,10 @@
         <v>1</v>
       </c>
       <c r="M145" t="n">
-        <v>-58.419652</v>
+        <v>-58.442098</v>
       </c>
       <c r="N145" t="n">
-        <v>-34.588271</v>
+        <v>-34.568762</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -12835,7 +12835,7 @@
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>VCR-K</t>
+          <t>BLO-G</t>
         </is>
       </c>
       <c r="R145" t="inlineStr">
@@ -12847,7 +12847,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>-775</t>
+          <t>-781</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -12857,7 +12857,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>11 DE SEPTIEMBRE DE 1888 996</t>
+          <t>ARENALES 3658</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -12872,7 +12872,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814125568</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
@@ -12892,7 +12892,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -12904,10 +12904,10 @@
         <v>1</v>
       </c>
       <c r="M146" t="n">
-        <v>-58.442098</v>
+        <v>-58.413717</v>
       </c>
       <c r="N146" t="n">
-        <v>-34.568762</v>
+        <v>-34.585425</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>BLO-G</t>
+          <t>AGU-L</t>
         </is>
       </c>
       <c r="R146" t="inlineStr">
@@ -12933,7 +12933,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>-781</t>
+          <t>-782</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -12943,7 +12943,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>ARENALES 3658</t>
+          <t>ARMENIA 1800</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -12958,7 +12958,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>814125568</t>
+          <t>814125577</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -12990,10 +12990,10 @@
         <v>1</v>
       </c>
       <c r="M147" t="n">
-        <v>-58.413717</v>
+        <v>-58.426328</v>
       </c>
       <c r="N147" t="n">
-        <v>-34.585425</v>
+        <v>-34.588734</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -13007,7 +13007,7 @@
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>AGU-L</t>
+          <t>VCR-F</t>
         </is>
       </c>
       <c r="R147" t="inlineStr">
@@ -13019,7 +13019,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>-782</t>
+          <t>-787</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -13029,7 +13029,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>ARMENIA 1800</t>
+          <t>CHENAUT, INDALESIO, GRAL. AV. 1945</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -13044,7 +13044,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>814125577</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -13064,7 +13064,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -13076,10 +13076,10 @@
         <v>1</v>
       </c>
       <c r="M148" t="n">
-        <v>-58.426328</v>
+        <v>-58.432822</v>
       </c>
       <c r="N148" t="n">
-        <v>-34.588734</v>
+        <v>-34.571917</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -13093,7 +13093,7 @@
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>VCR-F</t>
+          <t>BLO-H</t>
         </is>
       </c>
       <c r="R148" t="inlineStr">
@@ -13105,7 +13105,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>-787</t>
+          <t>-796</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -13115,7 +13115,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>CHENAUT, INDALESIO, GRAL. AV. 1945</t>
+          <t>CABRERA, JOSE A. 4723</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -13130,7 +13130,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814125624</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -13150,7 +13150,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -13162,10 +13162,10 @@
         <v>1</v>
       </c>
       <c r="M149" t="n">
-        <v>-58.432822</v>
+        <v>-58.429431</v>
       </c>
       <c r="N149" t="n">
-        <v>-34.571917</v>
+        <v>-34.591921</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -13179,7 +13179,7 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>BLO-H</t>
+          <t>VCR-F</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">
@@ -13191,7 +13191,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>-796</t>
+          <t>-797</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -13201,12 +13201,12 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>CABRERA, JOSE A. 4723</t>
+          <t>CHARCAS 3248</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
@@ -13216,7 +13216,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>814125624</t>
+          <t>814125633</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -13226,7 +13226,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>columna chocada</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -13248,14 +13248,14 @@
         <v>1</v>
       </c>
       <c r="M150" t="n">
-        <v>-58.429431</v>
+        <v>-58.411747</v>
       </c>
       <c r="N150" t="n">
-        <v>-34.591921</v>
+        <v>-34.592175</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P150" t="inlineStr">
@@ -13265,7 +13265,7 @@
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>VCR-F</t>
+          <t>AGU-C</t>
         </is>
       </c>
       <c r="R150" t="inlineStr">
@@ -13277,7 +13277,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>-797</t>
+          <t>-805</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -13287,12 +13287,12 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>CHARCAS 3248</t>
+          <t>MATIENZO, BENJAMIN, TENIENTE 1510</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -13302,7 +13302,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>814125633</t>
+          <t>814125656</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -13312,7 +13312,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>columna chocada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -13334,14 +13334,14 @@
         <v>1</v>
       </c>
       <c r="M151" t="n">
-        <v>-58.411747</v>
+        <v>-58.432345</v>
       </c>
       <c r="N151" t="n">
-        <v>-34.592175</v>
+        <v>-34.566345</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P151" t="inlineStr">
@@ -13351,7 +13351,7 @@
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>AGU-C</t>
+          <t>BLO-I</t>
         </is>
       </c>
       <c r="R151" t="inlineStr">
@@ -13363,22 +13363,22 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>-805</t>
+          <t>814446819</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>6/2/2026</t>
+          <t>6/11/2026</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>MATIENZO, BENJAMIN, TENIENTE 1510</t>
+          <t>ANGEL GALLARDO 946</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -13388,7 +13388,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>814125656</t>
+          <t>814446819</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -13398,7 +13398,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -13417,17 +13417,17 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M152" t="n">
-        <v>-58.432345</v>
+        <v>-58.443588</v>
       </c>
       <c r="N152" t="n">
-        <v>-34.566345</v>
+        <v>-34.606863</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P152" t="inlineStr">
@@ -13437,7 +13437,7 @@
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>BLO-I</t>
+          <t>ALM-O</t>
         </is>
       </c>
       <c r="R152" t="inlineStr">
@@ -13449,7 +13449,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>814446819</t>
+          <t>814446825</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -13459,7 +13459,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>ANGEL GALLARDO 946</t>
+          <t>ANGEL GALLARDO 1084</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -13474,7 +13474,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>814446819</t>
+          <t>814446825</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -13506,10 +13506,10 @@
         <v>0</v>
       </c>
       <c r="M153" t="n">
-        <v>-58.443588</v>
+        <v>-58.445084</v>
       </c>
       <c r="N153" t="n">
-        <v>-34.606863</v>
+        <v>-34.60725</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -13527,92 +13527,6 @@
         </is>
       </c>
       <c r="R153" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>814446825</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>6/11/2026</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>ANGEL GALLARDO 1084</t>
-        </is>
-      </c>
-      <c r="D154" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E154" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F154" t="inlineStr">
-        <is>
-          <t>814446825</t>
-        </is>
-      </c>
-      <c r="G154" t="inlineStr">
-        <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="H154" t="inlineStr">
-        <is>
-          <t>CAMBIAR COLUMNA</t>
-        </is>
-      </c>
-      <c r="I154" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J154" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K154" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L154" t="n">
-        <v>0</v>
-      </c>
-      <c r="M154" t="n">
-        <v>-58.445084</v>
-      </c>
-      <c r="N154" t="n">
-        <v>-34.60725</v>
-      </c>
-      <c r="O154" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="P154" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q154" t="inlineStr">
-        <is>
-          <t>ALM-O</t>
-        </is>
-      </c>
-      <c r="R154" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-28 09:49:24)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_PEBCOM.xlsx
+++ b/mapa_interactivo_PEBCOM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R153"/>
+  <dimension ref="A1:R152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11487,7 +11487,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t xml:space="preserve">9924 </t>
+          <t xml:space="preserve">10047 </t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -11497,7 +11497,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>CORDOBA AV. 4089</t>
+          <t>NEWBERY, JORGE 2410</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -11512,7 +11512,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>814108196</t>
+          <t>814111706</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -11522,7 +11522,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -11544,10 +11544,10 @@
         <v>1</v>
       </c>
       <c r="M130" t="n">
-        <v>-58.424553</v>
+        <v>-58.440973</v>
       </c>
       <c r="N130" t="n">
-        <v>-34.59709</v>
+        <v>-34.572415</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -11561,7 +11561,7 @@
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>VCR-D</t>
+          <t>COG-B</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
@@ -11573,7 +11573,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t xml:space="preserve">10047 </t>
+          <t>S01035299</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -11583,12 +11583,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>NEWBERY, JORGE 2410</t>
+          <t>ECUADOR 1390</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -11596,11 +11596,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F131" t="inlineStr">
-        <is>
-          <t>814111706</t>
-        </is>
-      </c>
+      <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -11613,12 +11609,12 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -11630,14 +11626,14 @@
         <v>1</v>
       </c>
       <c r="M131" t="n">
-        <v>-58.440973</v>
+        <v>-58.40382</v>
       </c>
       <c r="N131" t="n">
-        <v>-34.572415</v>
+        <v>-34.594385</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
@@ -11647,7 +11643,7 @@
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>COG-B</t>
+          <t>AGU-A</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
@@ -11659,7 +11655,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>S01035299</t>
+          <t xml:space="preserve">10042 </t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -11669,12 +11665,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>ECUADOR 1390</t>
+          <t>PARAGUAY 5310</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -11682,7 +11678,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F132" t="inlineStr"/>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>814108322</t>
+        </is>
+      </c>
       <c r="G132" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -11690,17 +11690,17 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -11712,14 +11712,14 @@
         <v>1</v>
       </c>
       <c r="M132" t="n">
-        <v>-58.40382</v>
+        <v>-58.43218</v>
       </c>
       <c r="N132" t="n">
-        <v>-34.594385</v>
+        <v>-34.578546</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P132" t="inlineStr">
@@ -11729,7 +11729,7 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>AGU-A</t>
+          <t>ATH-B</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
@@ -11741,7 +11741,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">10042 </t>
+          <t xml:space="preserve">10062 </t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>PARAGUAY 5310</t>
+          <t>HUMBOLDT 1556</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -11766,7 +11766,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>814108322</t>
+          <t>814108343</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
@@ -11798,10 +11798,10 @@
         <v>1</v>
       </c>
       <c r="M133" t="n">
-        <v>-58.43218</v>
+        <v>-58.436737</v>
       </c>
       <c r="N133" t="n">
-        <v>-34.578546</v>
+        <v>-34.58597</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -11815,7 +11815,7 @@
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>ATH-B</t>
+          <t>ATH-M</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
@@ -11827,7 +11827,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">10062 </t>
+          <t xml:space="preserve">10066 </t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -11837,7 +11837,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>HUMBOLDT 1556</t>
+          <t xml:space="preserve">ARENALES 3640 </t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -11850,11 +11850,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F134" t="inlineStr">
-        <is>
-          <t>814108343</t>
-        </is>
-      </c>
+      <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -11862,12 +11858,12 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>DESMONTAR COLUMNA</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -11884,10 +11880,10 @@
         <v>1</v>
       </c>
       <c r="M134" t="n">
-        <v>-58.436737</v>
+        <v>-58.413584</v>
       </c>
       <c r="N134" t="n">
-        <v>-34.58597</v>
+        <v>-34.58551</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -11901,7 +11897,7 @@
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>ATH-M</t>
+          <t>AGU-L</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
@@ -11913,7 +11909,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">10066 </t>
+          <t xml:space="preserve">10067 </t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -11923,7 +11919,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARENALES 3640 </t>
+          <t>CHARCAS 3601</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -11944,17 +11940,17 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>DESMONTAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -11966,10 +11962,10 @@
         <v>1</v>
       </c>
       <c r="M135" t="n">
-        <v>-58.413584</v>
+        <v>-58.415912</v>
       </c>
       <c r="N135" t="n">
-        <v>-34.58551</v>
+        <v>-34.588977</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -11983,7 +11979,7 @@
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>AGU-L</t>
+          <t>VCR-E</t>
         </is>
       </c>
       <c r="R135" t="inlineStr">
@@ -11995,7 +11991,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">10067 </t>
+          <t xml:space="preserve">10072 </t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -12005,7 +12001,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>CHARCAS 3601</t>
+          <t>SANTA FE AV. 3470</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -12018,7 +12014,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F136" t="inlineStr"/>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>814111751</t>
+        </is>
+      </c>
       <c r="G136" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -12031,12 +12031,12 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -12048,10 +12048,10 @@
         <v>1</v>
       </c>
       <c r="M136" t="n">
-        <v>-58.415912</v>
+        <v>-58.413885</v>
       </c>
       <c r="N136" t="n">
-        <v>-34.588977</v>
+        <v>-34.586628</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -12065,7 +12065,7 @@
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>VCR-E</t>
+          <t>VCR-G</t>
         </is>
       </c>
       <c r="R136" t="inlineStr">
@@ -12077,7 +12077,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">10072 </t>
+          <t xml:space="preserve">10082 </t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -12087,7 +12087,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>SANTA FE AV. 3470</t>
+          <t>TAGLE 2562</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>814111751</t>
+          <t>814108377</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
@@ -12112,7 +12112,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -12134,14 +12134,14 @@
         <v>1</v>
       </c>
       <c r="M137" t="n">
-        <v>-58.413885</v>
+        <v>-58.400188</v>
       </c>
       <c r="N137" t="n">
-        <v>-34.586628</v>
+        <v>-34.583882</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P137" t="inlineStr">
@@ -12151,7 +12151,7 @@
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>VCR-G</t>
+          <t>AGU-I</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
@@ -12163,7 +12163,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">10082 </t>
+          <t xml:space="preserve">10083 </t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -12173,7 +12173,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>TAGLE 2562</t>
+          <t>ORTIZ DE OCAMPO 2639</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -12188,7 +12188,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>814108377</t>
+          <t>814111784</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
@@ -12198,7 +12198,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -12220,10 +12220,10 @@
         <v>1</v>
       </c>
       <c r="M138" t="n">
-        <v>-58.400188</v>
+        <v>-58.404652</v>
       </c>
       <c r="N138" t="n">
-        <v>-34.583882</v>
+        <v>-34.58263</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -12237,7 +12237,7 @@
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>AGU-I</t>
+          <t>AGU-N</t>
         </is>
       </c>
       <c r="R138" t="inlineStr">
@@ -12249,7 +12249,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">10083 </t>
+          <t xml:space="preserve">10098 </t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -12259,7 +12259,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>ORTIZ DE OCAMPO 2639</t>
+          <t>DORREGO AV. 2635</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -12274,7 +12274,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>814111784</t>
+          <t>814108458</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -12284,7 +12284,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -12306,14 +12306,14 @@
         <v>1</v>
       </c>
       <c r="M139" t="n">
-        <v>-58.404652</v>
+        <v>-58.433857</v>
       </c>
       <c r="N139" t="n">
-        <v>-34.58263</v>
+        <v>-34.57424</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
@@ -12323,7 +12323,7 @@
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>AGU-N</t>
+          <t>BLO-G</t>
         </is>
       </c>
       <c r="R139" t="inlineStr">
@@ -12335,7 +12335,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">10098 </t>
+          <t xml:space="preserve">10103 </t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -12345,7 +12345,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>DORREGO AV. 2635</t>
+          <t>DORREGO AV. 2765</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -12360,7 +12360,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>814108458</t>
+          <t>814111791</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
@@ -12370,7 +12370,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -12392,10 +12392,10 @@
         <v>1</v>
       </c>
       <c r="M140" t="n">
-        <v>-58.433857</v>
+        <v>-58.432319</v>
       </c>
       <c r="N140" t="n">
-        <v>-34.57424</v>
+        <v>-34.574385</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -12421,7 +12421,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">10103 </t>
+          <t xml:space="preserve">10104 </t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -12431,7 +12431,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>DORREGO AV. 2765</t>
+          <t xml:space="preserve">DORREGO AV. 4050 </t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -12446,7 +12446,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>814111791</t>
+          <t>814108469</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -12456,7 +12456,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t xml:space="preserve">CAMBIAR COLUMNA </t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -12478,10 +12478,10 @@
         <v>1</v>
       </c>
       <c r="M141" t="n">
-        <v>-58.432319</v>
+        <v>-58.416882</v>
       </c>
       <c r="N141" t="n">
-        <v>-34.574385</v>
+        <v>-34.562655</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -12495,7 +12495,7 @@
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>BLO-G</t>
+          <t>BLO-?</t>
         </is>
       </c>
       <c r="R141" t="inlineStr">
@@ -12507,7 +12507,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">10104 </t>
+          <t xml:space="preserve">10129 </t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -12517,7 +12517,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t xml:space="preserve">DORREGO AV. 4050 </t>
+          <t>ALVAREZ, JULIAN 1890</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -12532,7 +12532,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>814108469</t>
+          <t>814111804</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
@@ -12542,7 +12542,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAMBIAR COLUMNA </t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -12557,17 +12557,17 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L142" t="n">
         <v>1</v>
       </c>
       <c r="M142" t="n">
-        <v>-58.416882</v>
+        <v>-58.42056</v>
       </c>
       <c r="N142" t="n">
-        <v>-34.562655</v>
+        <v>-34.590217</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -12581,7 +12581,7 @@
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>BLO-?</t>
+          <t>VCR-D</t>
         </is>
       </c>
       <c r="R142" t="inlineStr">
@@ -12593,7 +12593,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">10129 </t>
+          <t xml:space="preserve">10131 </t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -12603,7 +12603,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>ALVAREZ, JULIAN 1890</t>
+          <t xml:space="preserve">PARAGUAY 4022 </t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -12616,11 +12616,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F143" t="inlineStr">
-        <is>
-          <t>814111804</t>
-        </is>
-      </c>
+      <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -12628,7 +12624,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -12638,22 +12634,22 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L143" t="n">
         <v>1</v>
       </c>
       <c r="M143" t="n">
-        <v>-58.42056</v>
+        <v>-58.419652</v>
       </c>
       <c r="N143" t="n">
-        <v>-34.590217</v>
+        <v>-34.588271</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -12667,7 +12663,7 @@
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>VCR-D</t>
+          <t>VCR-K</t>
         </is>
       </c>
       <c r="R143" t="inlineStr">
@@ -12679,17 +12675,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">10131 </t>
+          <t>-775</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>6/2/2026</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t xml:space="preserve">PARAGUAY 4022 </t>
+          <t>11 DE SEPTIEMBRE DE 1888 996</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -12702,7 +12698,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F144" t="inlineStr"/>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
       <c r="G144" t="inlineStr">
         <is>
           <t>PEBCOM</t>
@@ -12710,7 +12710,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -12720,7 +12720,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -12732,10 +12732,10 @@
         <v>1</v>
       </c>
       <c r="M144" t="n">
-        <v>-58.419652</v>
+        <v>-58.442098</v>
       </c>
       <c r="N144" t="n">
-        <v>-34.588271</v>
+        <v>-34.568762</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -12749,7 +12749,7 @@
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>VCR-K</t>
+          <t>BLO-G</t>
         </is>
       </c>
       <c r="R144" t="inlineStr">
@@ -12761,7 +12761,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>-775</t>
+          <t>-781</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -12771,7 +12771,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>11 DE SEPTIEMBRE DE 1888 996</t>
+          <t>ARENALES 3658</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -12786,7 +12786,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814125568</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -12818,10 +12818,10 @@
         <v>1</v>
       </c>
       <c r="M145" t="n">
-        <v>-58.442098</v>
+        <v>-58.413717</v>
       </c>
       <c r="N145" t="n">
-        <v>-34.568762</v>
+        <v>-34.585425</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -12835,7 +12835,7 @@
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>BLO-G</t>
+          <t>AGU-L</t>
         </is>
       </c>
       <c r="R145" t="inlineStr">
@@ -12847,7 +12847,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>-781</t>
+          <t>-782</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -12857,7 +12857,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>ARENALES 3658</t>
+          <t>ARMENIA 1800</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -12872,7 +12872,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>814125568</t>
+          <t>814125577</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
@@ -12904,10 +12904,10 @@
         <v>1</v>
       </c>
       <c r="M146" t="n">
-        <v>-58.413717</v>
+        <v>-58.426328</v>
       </c>
       <c r="N146" t="n">
-        <v>-34.585425</v>
+        <v>-34.588734</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>AGU-L</t>
+          <t>VCR-F</t>
         </is>
       </c>
       <c r="R146" t="inlineStr">
@@ -12933,7 +12933,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>-782</t>
+          <t>-787</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -12943,7 +12943,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>ARMENIA 1800</t>
+          <t>CHENAUT, INDALESIO, GRAL. AV. 1945</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -12958,7 +12958,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>814125577</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -12978,7 +12978,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -12990,10 +12990,10 @@
         <v>1</v>
       </c>
       <c r="M147" t="n">
-        <v>-58.426328</v>
+        <v>-58.432822</v>
       </c>
       <c r="N147" t="n">
-        <v>-34.588734</v>
+        <v>-34.571917</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -13007,7 +13007,7 @@
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>VCR-F</t>
+          <t>BLO-H</t>
         </is>
       </c>
       <c r="R147" t="inlineStr">
@@ -13019,7 +13019,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>-787</t>
+          <t>-796</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -13029,7 +13029,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>CHENAUT, INDALESIO, GRAL. AV. 1945</t>
+          <t>CABRERA, JOSE A. 4723</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -13044,7 +13044,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814125624</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -13064,7 +13064,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -13076,10 +13076,10 @@
         <v>1</v>
       </c>
       <c r="M148" t="n">
-        <v>-58.432822</v>
+        <v>-58.429431</v>
       </c>
       <c r="N148" t="n">
-        <v>-34.571917</v>
+        <v>-34.591921</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -13093,7 +13093,7 @@
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>BLO-H</t>
+          <t>VCR-F</t>
         </is>
       </c>
       <c r="R148" t="inlineStr">
@@ -13105,7 +13105,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>-796</t>
+          <t>-797</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -13115,12 +13115,12 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>CABRERA, JOSE A. 4723</t>
+          <t>CHARCAS 3248</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -13130,7 +13130,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>814125624</t>
+          <t>814125633</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -13140,7 +13140,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>columna chocada</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -13162,14 +13162,14 @@
         <v>1</v>
       </c>
       <c r="M149" t="n">
-        <v>-58.429431</v>
+        <v>-58.411747</v>
       </c>
       <c r="N149" t="n">
-        <v>-34.591921</v>
+        <v>-34.592175</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P149" t="inlineStr">
@@ -13179,7 +13179,7 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>VCR-F</t>
+          <t>AGU-C</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">
@@ -13191,7 +13191,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>-797</t>
+          <t>-805</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -13201,12 +13201,12 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>CHARCAS 3248</t>
+          <t>MATIENZO, BENJAMIN, TENIENTE 1510</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
@@ -13216,7 +13216,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>814125633</t>
+          <t>814125656</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -13226,7 +13226,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>columna chocada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -13248,14 +13248,14 @@
         <v>1</v>
       </c>
       <c r="M150" t="n">
-        <v>-58.411747</v>
+        <v>-58.432345</v>
       </c>
       <c r="N150" t="n">
-        <v>-34.592175</v>
+        <v>-34.566345</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P150" t="inlineStr">
@@ -13265,7 +13265,7 @@
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>AGU-C</t>
+          <t>BLO-I</t>
         </is>
       </c>
       <c r="R150" t="inlineStr">
@@ -13277,22 +13277,22 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>-805</t>
+          <t>814446819</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>6/2/2026</t>
+          <t>6/11/2026</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>MATIENZO, BENJAMIN, TENIENTE 1510</t>
+          <t>ANGEL GALLARDO 946</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -13302,7 +13302,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>814125656</t>
+          <t>814446819</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -13312,7 +13312,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -13331,17 +13331,17 @@
         </is>
       </c>
       <c r="L151" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M151" t="n">
-        <v>-58.432345</v>
+        <v>-58.443588</v>
       </c>
       <c r="N151" t="n">
-        <v>-34.566345</v>
+        <v>-34.606863</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P151" t="inlineStr">
@@ -13351,7 +13351,7 @@
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>BLO-I</t>
+          <t>ALM-O</t>
         </is>
       </c>
       <c r="R151" t="inlineStr">
@@ -13363,7 +13363,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>814446819</t>
+          <t>814446825</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -13373,7 +13373,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>ANGEL GALLARDO 946</t>
+          <t>ANGEL GALLARDO 1084</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -13388,7 +13388,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>814446819</t>
+          <t>814446825</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -13420,10 +13420,10 @@
         <v>0</v>
       </c>
       <c r="M152" t="n">
-        <v>-58.443588</v>
+        <v>-58.445084</v>
       </c>
       <c r="N152" t="n">
-        <v>-34.606863</v>
+        <v>-34.60725</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -13441,92 +13441,6 @@
         </is>
       </c>
       <c r="R152" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>814446825</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>6/11/2026</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>ANGEL GALLARDO 1084</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E153" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F153" t="inlineStr">
-        <is>
-          <t>814446825</t>
-        </is>
-      </c>
-      <c r="G153" t="inlineStr">
-        <is>
-          <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="H153" t="inlineStr">
-        <is>
-          <t>CAMBIAR COLUMNA</t>
-        </is>
-      </c>
-      <c r="I153" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J153" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K153" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L153" t="n">
-        <v>0</v>
-      </c>
-      <c r="M153" t="n">
-        <v>-58.445084</v>
-      </c>
-      <c r="N153" t="n">
-        <v>-34.60725</v>
-      </c>
-      <c r="O153" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="P153" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q153" t="inlineStr">
-        <is>
-          <t>ALM-O</t>
-        </is>
-      </c>
-      <c r="R153" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>